<commit_message>
Fix bet history with matchup season CLV
</commit_message>
<xml_diff>
--- a/WebsiteData.xlsx
+++ b/WebsiteData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkevans/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F61EA5D-A4DD-9846-B64D-AF1C35AA234F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACC96171-BDE1-4147-A4AC-21721A12FFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="840" windowWidth="26480" windowHeight="20020" activeTab="1" xr2:uid="{C762ECBC-EE1A-4249-820F-B10BC232F997}"/>
+    <workbookView xWindow="0" yWindow="840" windowWidth="17200" windowHeight="20020" activeTab="1" xr2:uid="{C762ECBC-EE1A-4249-820F-B10BC232F997}"/>
   </bookViews>
   <sheets>
     <sheet name="Projections" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="440">
   <si>
     <t>Team</t>
   </si>
@@ -1338,6 +1338,33 @@
   </si>
   <si>
     <t>03/12/2026</t>
+  </si>
+  <si>
+    <t>03/13/2026</t>
+  </si>
+  <si>
+    <t>Matchup</t>
+  </si>
+  <si>
+    <t>MST/LT</t>
+  </si>
+  <si>
+    <t>TENN/VAN</t>
+  </si>
+  <si>
+    <t>DAV/LOY</t>
+  </si>
+  <si>
+    <t>XU/MARQ</t>
+  </si>
+  <si>
+    <t>WAKE/VT</t>
+  </si>
+  <si>
+    <t>WEB/EWASH</t>
+  </si>
+  <si>
+    <t>ILL/MD</t>
   </si>
 </sst>
 </file>
@@ -26069,7 +26096,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B49754F4-77C8-5D43-B0D7-0D09062FB370}">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="1"/>
@@ -26077,14 +26104,14 @@
     <col min="4" max="4" width="13" style="1" customWidth="1"/>
     <col min="5" max="5" width="11.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.33203125" customWidth="1"/>
-    <col min="11" max="11" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" customWidth="1"/>
+    <col min="12" max="12" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>388</v>
       </c>
@@ -26105,31 +26132,31 @@
       </c>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <f>COUNTIF($C$6:$C$150,"W")</f>
         <v>2</v>
       </c>
       <c r="B2" s="1">
         <f>COUNTIF($C$6:$C$150,"L")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C2" s="13">
-        <f>SUM(E6:E13)/SUM(D6:D13)</f>
-        <v>-0.37626460284041197</v>
+        <f>SUM(F6:F13)/SUM(E6:E13)</f>
+        <v>-0.52691906581309589</v>
       </c>
       <c r="D2" s="14">
-        <f>AVERAGE(G6:G150)</f>
-        <v>1.2346518407494022E-2</v>
+        <f>AVERAGE(H6:H150)</f>
+        <v>4.1788135989584758E-2</v>
       </c>
       <c r="E2" s="1">
         <v>2</v>
       </c>
       <c r="F2" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>394</v>
       </c>
@@ -26140,40 +26167,46 @@
         <v>398</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="P5" s="1" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>424</v>
       </c>
@@ -26183,47 +26216,53 @@
       <c r="C6" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="E6" s="1">
         <v>0.94499999999999995</v>
       </c>
-      <c r="E6" s="15">
-        <f>IF(C6="P",0,IF(C6="L",-D6,IF(I6&lt;0,D6*(100/-I6),D6*(I6/100)))/1)</f>
+      <c r="F6" s="15">
+        <f>IF(C6="P",0,IF(C6="L",-E6,IF(K6&lt;0,E6*(100/-K6),E6*(K6/100)))/1)</f>
         <v>-0.94499999999999995</v>
       </c>
-      <c r="F6" s="15">
-        <f>E6</f>
+      <c r="G6" s="15">
+        <f>F6</f>
         <v>-0.94499999999999995</v>
       </c>
-      <c r="G6" s="11">
-        <f>((K6-N6)*3.55%)+(M6-J6)</f>
+      <c r="H6" s="11">
+        <f>((M6-P6)*3.55%)+(O6-L6)</f>
         <v>-1.9985536081552357E-2</v>
       </c>
-      <c r="H6" s="11">
-        <f>G6</f>
+      <c r="I6" s="11">
+        <f>H6</f>
         <v>-1.9985536081552357E-2</v>
       </c>
-      <c r="I6" s="1">
+      <c r="J6" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="K6" s="1">
         <v>-112</v>
       </c>
-      <c r="J6" s="13">
-        <f>IF(I6&lt;0,I6/(I6-100),100/(I6+100))</f>
+      <c r="L6" s="13">
+        <f>IF(K6&lt;0,K6/(K6-100),100/(K6+100))</f>
         <v>0.52830188679245282</v>
       </c>
-      <c r="K6" s="1">
+      <c r="M6" s="1">
         <v>-14.5</v>
       </c>
-      <c r="L6" s="1">
+      <c r="N6" s="1">
         <v>-111</v>
       </c>
-      <c r="M6" s="13">
-        <f>IF(L6&lt;0,L6/(L6-100),100/(L6+100))</f>
+      <c r="O6" s="13">
+        <f>IF(N6&lt;0,N6/(N6-100),100/(N6+100))</f>
         <v>0.52606635071090047</v>
       </c>
-      <c r="N6" s="1">
+      <c r="P6" s="1">
         <v>-14</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>426</v>
       </c>
@@ -26233,47 +26272,53 @@
       <c r="C7" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="E7" s="1">
         <v>0.68979999999999997</v>
       </c>
-      <c r="E7" s="15">
-        <f>IF(C7="P",0,IF(C7="L",-D7,IF(I7&lt;0,D7*(100/-I7),D7*(I7/100)))/1)</f>
+      <c r="F7" s="15">
+        <f>IF(C7="P",0,IF(C7="L",-E7,IF(K7&lt;0,E7*(100/-K7),E7*(K7/100)))/1)</f>
         <v>-0.68979999999999997</v>
       </c>
-      <c r="F7" s="15">
-        <f>E7+F6</f>
+      <c r="G7" s="15">
+        <f>F7+G6</f>
         <v>-1.6347999999999998</v>
       </c>
-      <c r="G7" s="11">
-        <f>((K7-N7)*3.55%)+(M7-J7)</f>
+      <c r="H7" s="11">
+        <f>((M7-P7)*3.55%)+(O7-L7)</f>
         <v>5.3772693633062259E-3</v>
       </c>
-      <c r="H7" s="11">
-        <f>AVERAGE($G$6:G7)</f>
+      <c r="I7" s="11">
+        <f>AVERAGE($H$6:H7)</f>
         <v>-7.3041333591230655E-3</v>
       </c>
-      <c r="I7" s="1">
+      <c r="J7" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="K7" s="1">
         <v>-103</v>
       </c>
-      <c r="J7" s="13">
-        <f>IF(I7&lt;0,I7/(I7-100),100/(I7+100))</f>
+      <c r="L7" s="13">
+        <f>IF(K7&lt;0,K7/(K7-100),100/(K7+100))</f>
         <v>0.5073891625615764</v>
       </c>
-      <c r="K7" s="1">
+      <c r="M7" s="1">
         <v>3</v>
       </c>
-      <c r="L7" s="1">
+      <c r="N7" s="1">
         <v>-113</v>
       </c>
-      <c r="M7" s="13">
-        <f>IF(L7&lt;0,L7/(L7-100),100/(L7+100))</f>
+      <c r="O7" s="13">
+        <f>IF(N7&lt;0,N7/(N7-100),100/(N7+100))</f>
         <v>0.53051643192488263</v>
       </c>
-      <c r="N7" s="1">
+      <c r="P7" s="1">
         <v>3.5</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>427</v>
       </c>
@@ -26283,47 +26328,53 @@
       <c r="C8" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="E8" s="1">
         <v>0.74019999999999997</v>
       </c>
-      <c r="E8" s="15">
-        <f>IF(C8="P",0,IF(C8="L",-D8,IF(I8&lt;0,D8*(100/-I8),D8*(I8/100)))/1)</f>
+      <c r="F8" s="15">
+        <f>IF(C8="P",0,IF(C8="L",-E8,IF(K8&lt;0,E8*(100/-K8),E8*(K8/100)))/1)</f>
         <v>0.6729090909090909</v>
       </c>
-      <c r="F8" s="15">
-        <f>E8+F7</f>
+      <c r="G8" s="15">
+        <f>F8+G7</f>
         <v>-0.96189090909090891</v>
       </c>
-      <c r="G8" s="11">
-        <f>((K8-N8)*3.55%)+(M8-J8)</f>
+      <c r="H8" s="11">
+        <f>((M8-P8)*3.55%)+(O8-L8)</f>
         <v>0.10782963875205255</v>
       </c>
-      <c r="H8" s="11">
-        <f>AVERAGE($G$6:G8)</f>
+      <c r="I8" s="11">
+        <f>AVERAGE($H$6:H8)</f>
         <v>3.1073790677935476E-2</v>
       </c>
-      <c r="I8" s="1">
+      <c r="J8" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="K8" s="1">
         <v>-110</v>
       </c>
-      <c r="J8" s="13">
-        <f>IF(I8&lt;0,I8/(I8-100),100/(I8+100))</f>
+      <c r="L8" s="13">
+        <f>IF(K8&lt;0,K8/(K8-100),100/(K8+100))</f>
         <v>0.52380952380952384</v>
       </c>
-      <c r="K8" s="1">
+      <c r="M8" s="1">
         <v>2.5</v>
       </c>
-      <c r="L8" s="1">
+      <c r="N8" s="1">
         <v>-103</v>
       </c>
-      <c r="M8" s="13">
-        <f>IF(L8&lt;0,L8/(L8-100),100/(L8+100))</f>
+      <c r="O8" s="13">
+        <f>IF(N8&lt;0,N8/(N8-100),100/(N8+100))</f>
         <v>0.5073891625615764</v>
       </c>
-      <c r="N8" s="1">
+      <c r="P8" s="1">
         <v>-1</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>429</v>
       </c>
@@ -26333,47 +26384,53 @@
       <c r="C9" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="E9" s="1">
         <v>0.67900000000000005</v>
       </c>
-      <c r="E9" s="15">
-        <f>IF(C9="P",0,IF(C9="L",-D9,IF(I9&lt;0,D9*(100/-I9),D9*(I9/100)))/1)</f>
+      <c r="F9" s="15">
+        <f>IF(C9="P",0,IF(C9="L",-E9,IF(K9&lt;0,E9*(100/-K9),E9*(K9/100)))/1)</f>
         <v>0.61727272727272731</v>
       </c>
-      <c r="F9" s="15">
-        <f>E9+F8</f>
+      <c r="G9" s="15">
+        <f>F9+G8</f>
         <v>-0.3446181818181816</v>
       </c>
-      <c r="G9" s="11">
-        <f>((K9-N9)*3.55%)+(M9-J9)</f>
+      <c r="H9" s="11">
+        <f>((M9-P9)*3.55%)+(O9-L9)</f>
         <v>8.5035829865926608E-3</v>
       </c>
-      <c r="H9" s="11">
-        <f>AVERAGE($G$6:G9)</f>
+      <c r="I9" s="11">
+        <f>AVERAGE($H$6:H9)</f>
         <v>2.5431238755099773E-2</v>
       </c>
-      <c r="I9" s="1">
+      <c r="J9" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="K9" s="1">
         <v>-110</v>
       </c>
-      <c r="J9" s="13">
-        <f>IF(I9&lt;0,I9/(I9-100),100/(I9+100))</f>
+      <c r="L9" s="13">
+        <f>IF(K9&lt;0,K9/(K9-100),100/(K9+100))</f>
         <v>0.52380952380952384</v>
       </c>
-      <c r="K9" s="1">
+      <c r="M9" s="1">
         <v>4.5</v>
       </c>
-      <c r="L9" s="1">
+      <c r="N9" s="1">
         <v>-106</v>
       </c>
-      <c r="M9" s="13">
-        <f>IF(L9&lt;0,L9/(L9-100),100/(L9+100))</f>
+      <c r="O9" s="13">
+        <f>IF(N9&lt;0,N9/(N9-100),100/(N9+100))</f>
         <v>0.5145631067961165</v>
       </c>
-      <c r="N9" s="1">
+      <c r="P9" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>430</v>
       </c>
@@ -26383,45 +26440,185 @@
       <c r="C10" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="E10" s="1">
         <v>1.2898000000000001</v>
       </c>
-      <c r="E10" s="15">
-        <f>IF(C10="P",0,IF(C10="L",-D10,IF(I10&lt;0,D10*(100/-I10),D10*(I10/100)))/1)</f>
+      <c r="F10" s="15">
+        <f>IF(C10="P",0,IF(C10="L",-E10,IF(K10&lt;0,E10*(100/-K10),E10*(K10/100)))/1)</f>
         <v>-1.2898000000000001</v>
       </c>
-      <c r="F10" s="15">
-        <f>E10+F9</f>
+      <c r="G10" s="15">
+        <f>F10+G9</f>
         <v>-1.6344181818181815</v>
       </c>
-      <c r="G10" s="11">
-        <f>((K10-N10)*3.55%)+(M10-J10)</f>
+      <c r="H10" s="11">
+        <f>((M10-P10)*3.55%)+(O10-L10)</f>
         <v>-3.9992362982928985E-2</v>
       </c>
-      <c r="H10" s="11">
-        <f>AVERAGE($G$6:G10)</f>
+      <c r="I10" s="11">
+        <f>AVERAGE($H$6:H10)</f>
         <v>1.2346518407494022E-2</v>
       </c>
-      <c r="I10" s="1">
+      <c r="J10" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="K10" s="1">
         <v>-112</v>
       </c>
-      <c r="J10" s="13">
-        <f>IF(I10&lt;0,I10/(I10-100),100/(I10+100))</f>
+      <c r="L10" s="13">
+        <f>IF(K10&lt;0,K10/(K10-100),100/(K10+100))</f>
         <v>0.52830188679245282</v>
       </c>
-      <c r="K10" s="1">
+      <c r="M10" s="1">
         <v>-6.5</v>
       </c>
-      <c r="L10" s="1">
+      <c r="N10" s="1">
         <v>-110</v>
       </c>
-      <c r="M10" s="13">
-        <f>IF(L10&lt;0,L10/(L10-100),100/(L10+100))</f>
+      <c r="O10" s="13">
+        <f>IF(N10&lt;0,N10/(N10-100),100/(N10+100))</f>
         <v>0.52380952380952384</v>
       </c>
-      <c r="N10" s="1">
+      <c r="P10" s="1">
         <v>-5.5</v>
       </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B11" s="1">
+        <v>6</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.68820000000000003</v>
+      </c>
+      <c r="F11" s="15">
+        <f>IF(C11="P",0,IF(C11="L",-E11,IF(K11&lt;0,E11*(100/-K11),E11*(K11/100)))/1)</f>
+        <v>-0.68820000000000003</v>
+      </c>
+      <c r="G11" s="15">
+        <f t="shared" ref="G11:G12" si="0">F11+G10</f>
+        <v>-2.3226181818181817</v>
+      </c>
+      <c r="H11" s="11">
+        <f>((M11-P11)*3.55%)+(O11-L11)</f>
+        <v>9.1028423331054986E-2</v>
+      </c>
+      <c r="I11" s="11">
+        <f>AVERAGE($H$6:H11)</f>
+        <v>2.5460169228087515E-2</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="K11" s="1">
+        <v>-109</v>
+      </c>
+      <c r="L11" s="13">
+        <f>IF(K11&lt;0,K11/(K11-100),100/(K11+100))</f>
+        <v>0.52153110047846885</v>
+      </c>
+      <c r="M11" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="N11" s="1">
+        <v>-110</v>
+      </c>
+      <c r="O11" s="13">
+        <f>IF(N11&lt;0,N11/(N11-100),100/(N11+100))</f>
+        <v>0.52380952380952384</v>
+      </c>
+      <c r="P11" s="1">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B12" s="1">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.69510000000000005</v>
+      </c>
+      <c r="F12" s="15">
+        <f>IF(C12="P",0,IF(C12="L",-E12,IF(K12&lt;0,E12*(100/-K12),E12*(K12/100)))/1)</f>
+        <v>-0.69510000000000005</v>
+      </c>
+      <c r="G12" s="15">
+        <f t="shared" si="0"/>
+        <v>-3.0177181818181817</v>
+      </c>
+      <c r="H12" s="11">
+        <f>((M12-P12)*3.55%)+(O12-L12)</f>
+        <v>0.13975593655856822</v>
+      </c>
+      <c r="I12" s="11">
+        <f>AVERAGE($H$6:H12)</f>
+        <v>4.1788135989584758E-2</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="K12" s="1">
+        <v>-109</v>
+      </c>
+      <c r="L12" s="13">
+        <f>IF(K12&lt;0,K12/(K12-100),100/(K12+100))</f>
+        <v>0.52153110047846885</v>
+      </c>
+      <c r="M12" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="N12" s="1">
+        <v>-116</v>
+      </c>
+      <c r="O12" s="13">
+        <f>IF(N12&lt;0,N12/(N12-100),100/(N12+100))</f>
+        <v>0.53703703703703709</v>
+      </c>
+      <c r="P12" s="1">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="1"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I16" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add show projections flag
</commit_message>
<xml_diff>
--- a/WebsiteData.xlsx
+++ b/WebsiteData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkevans/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA8CC556-3375-F144-BE0D-9972CD86E05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D37BB91C-3606-1347-8863-5D322282D70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="27580" windowHeight="20000" activeTab="1" xr2:uid="{C762ECBC-EE1A-4249-820F-B10BC232F997}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="27580" windowHeight="20000" xr2:uid="{C762ECBC-EE1A-4249-820F-B10BC232F997}"/>
   </bookViews>
   <sheets>
     <sheet name="Projections" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="443">
   <si>
     <t>Team</t>
   </si>
@@ -1226,9 +1226,6 @@
     <t>Bet</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -1329,9 +1326,6 @@
   </si>
   <si>
     <t>03/10/2026</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>03/11/2026</t>
@@ -24201,7 +24195,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2A118F-D7F3-5348-BECB-A41992F5CAD2}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -24225,13 +24219,13 @@
         <v>368</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>369</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>370</v>
@@ -24250,224 +24244,79 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>4</v>
-      </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="6" t="e">
         <f>VLOOKUP(A2,[1]Games!$B$2:$K$398,2,FALSE)</f>
-        <v>VCU</v>
-      </c>
-      <c r="C2" s="6" t="str">
+        <v>#N/A</v>
+      </c>
+      <c r="C2" s="6" t="e">
         <f>VLOOKUP(A2,[1]Games!$B$2:$K$398,3,FALSE)</f>
-        <v>St. Joseph's</v>
-      </c>
-      <c r="D2" s="6" t="str">
+        <v>#N/A</v>
+      </c>
+      <c r="D2" s="6" t="e">
         <f>B2</f>
-        <v>VCU</v>
-      </c>
-      <c r="E2" s="5">
+        <v>#N/A</v>
+      </c>
+      <c r="E2" s="5" t="e">
         <f>VLOOKUP(A2,[1]Games!$B$2:$K$398,4,FALSE)</f>
-        <v>12.835404558957849</v>
-      </c>
-      <c r="F2" s="5">
+        <v>#N/A</v>
+      </c>
+      <c r="F2" s="5" t="e">
         <f>-VLOOKUP(A2,[2]Games!$A$2:$X$300,24,FALSE)</f>
-        <v>6</v>
-      </c>
-      <c r="G2" s="7">
+        <v>#N/A</v>
+      </c>
+      <c r="G2" s="7" t="e">
         <f>VLOOKUP(A2,[1]Games!$B$2:$K$398,9,FALSE)</f>
-        <v>0.70074839245243137</v>
-      </c>
-      <c r="H2" s="7">
+        <v>#N/A</v>
+      </c>
+      <c r="H2" s="7" t="e">
         <f>VLOOKUP(A2,[1]Games!$B$2:$K$398,7,FALSE)</f>
-        <v>7.0887631768342563E-2</v>
-      </c>
-      <c r="I2" s="7">
+        <v>#N/A</v>
+      </c>
+      <c r="I2" s="7" t="e">
         <f>VLOOKUP(A2,[1]Games!$B$2:$K$398,8,FALSE)/4</f>
-        <v>5.732251805019465E-2</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>393</v>
-      </c>
+        <v>#N/A</v>
+      </c>
+      <c r="J2" s="8"/>
       <c r="K2" s="9">
         <f>IF(J2="Yes",(H2*1500)/100,0)</f>
-        <v>1.0633144765251386</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>8</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <f>VLOOKUP(A3,[1]Games!$B$2:$K$398,2,FALSE)</f>
-        <v>Arkansas</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <f>VLOOKUP(A3,[1]Games!$B$2:$K$398,3,FALSE)</f>
-        <v>Ole Miss</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <f t="shared" ref="D3" si="0">B3</f>
-        <v>Arkansas</v>
-      </c>
-      <c r="E3" s="5">
-        <f>VLOOKUP(A3,[1]Games!$B$2:$K$398,4,FALSE)</f>
-        <v>14.94229486295097</v>
-      </c>
-      <c r="F3" s="5">
-        <f>-VLOOKUP(A3,[2]Games!$A$2:$X$300,24,FALSE)</f>
-        <v>9</v>
-      </c>
-      <c r="G3" s="7">
-        <f>VLOOKUP(A3,[1]Games!$B$2:$K$398,9,FALSE)</f>
-        <v>0.70816933596251053</v>
-      </c>
-      <c r="H3" s="7">
-        <f>VLOOKUP(A3,[1]Games!$B$2:$K$398,7,FALSE)</f>
-        <v>5.5077610628663218E-2</v>
-      </c>
-      <c r="I3" s="7">
-        <f>VLOOKUP(A3,[1]Games!$B$2:$K$398,8,FALSE)/4</f>
-        <v>4.8339551493558675E-2</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>393</v>
-      </c>
-      <c r="K3" s="9">
-        <f t="shared" ref="K3" si="1">IF(J3="Yes",(H3*1500)/100,0)</f>
-        <v>0.82616415942994825</v>
-      </c>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="10"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>15</v>
-      </c>
-      <c r="B4" s="6" t="str">
-        <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,2,FALSE)</f>
-        <v>Duke</v>
-      </c>
-      <c r="C4" s="6" t="str">
-        <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,3,FALSE)</f>
-        <v>Virginia</v>
-      </c>
-      <c r="D4" s="6" t="str">
-        <f t="shared" ref="D4:D6" si="2">B4</f>
-        <v>Duke</v>
-      </c>
-      <c r="E4" s="5">
-        <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,4,FALSE)</f>
-        <v>15.61990006839136</v>
-      </c>
-      <c r="F4" s="5">
-        <f>-VLOOKUP(A4,[2]Games!$A$2:$X$300,24,FALSE)</f>
-        <v>8.5</v>
-      </c>
-      <c r="G4" s="7">
-        <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,9,FALSE)</f>
-        <v>0.75149652484483553</v>
-      </c>
-      <c r="H4" s="7">
-        <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,7,FALSE)</f>
-        <v>7.0744352533153906E-2</v>
-      </c>
-      <c r="I4" s="7">
-        <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,8,FALSE)/4</f>
-        <v>5.7241109393837447E-2</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>428</v>
-      </c>
-      <c r="K4" s="9">
-        <f t="shared" ref="K4:K6" si="3">IF(J4="Yes",(H4*1500)/100,0)</f>
-        <v>0</v>
-      </c>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="10"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>23</v>
-      </c>
-      <c r="B5" s="6" t="str">
-        <f>VLOOKUP(A5,[1]Games!$B$2:$K$398,2,FALSE)</f>
-        <v>Pennsylvania</v>
-      </c>
-      <c r="C5" s="6" t="str">
-        <f>VLOOKUP(A5,[1]Games!$B$2:$K$398,3,FALSE)</f>
-        <v>Harvard</v>
-      </c>
-      <c r="D5" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v>Pennsylvania</v>
-      </c>
-      <c r="E5" s="5">
-        <f>VLOOKUP(A5,[1]Games!$B$2:$K$398,4,FALSE)</f>
-        <v>2.236546994210157</v>
-      </c>
-      <c r="F5" s="5">
-        <f>-VLOOKUP(A5,[2]Games!$A$2:$X$300,24,FALSE)</f>
-        <v>-3.5</v>
-      </c>
-      <c r="G5" s="7">
-        <f>VLOOKUP(A5,[1]Games!$B$2:$K$398,9,FALSE)</f>
-        <v>0.40688974186433241</v>
-      </c>
-      <c r="H5" s="7">
-        <f>VLOOKUP(A5,[1]Games!$B$2:$K$398,7,FALSE)</f>
-        <v>6.7623692875932173E-2</v>
-      </c>
-      <c r="I5" s="7">
-        <f>VLOOKUP(A5,[1]Games!$B$2:$K$398,8,FALSE)/4</f>
-        <v>5.54680073158706E-2</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>428</v>
-      </c>
-      <c r="K5" s="9">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="10"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>37</v>
-      </c>
-      <c r="B6" s="6" t="str">
-        <f>VLOOKUP(A6,[1]Games!$B$2:$K$398,2,FALSE)</f>
-        <v>Kennesaw State</v>
-      </c>
-      <c r="C6" s="6" t="str">
-        <f>VLOOKUP(A6,[1]Games!$B$2:$K$398,3,FALSE)</f>
-        <v>Louisiana Tech</v>
-      </c>
-      <c r="D6" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v>Kennesaw State</v>
-      </c>
-      <c r="E6" s="5">
-        <f>VLOOKUP(A6,[1]Games!$B$2:$K$398,4,FALSE)</f>
-        <v>6.2621855083836948</v>
-      </c>
-      <c r="F6" s="5">
-        <f>-VLOOKUP(A6,[2]Games!$A$2:$X$300,24,FALSE)</f>
-        <v>1.5</v>
-      </c>
-      <c r="G6" s="7">
-        <f>VLOOKUP(A6,[1]Games!$B$2:$K$398,9,FALSE)</f>
-        <v>0.47249844996534662</v>
-      </c>
-      <c r="H6" s="7">
-        <f>VLOOKUP(A6,[1]Games!$B$2:$K$398,7,FALSE)</f>
-        <v>4.8136336457088799E-2</v>
-      </c>
-      <c r="I6" s="7">
-        <f>VLOOKUP(A6,[1]Games!$B$2:$K$398,8,FALSE)/4</f>
-        <v>4.4395645714254972E-2</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>393</v>
-      </c>
-      <c r="K6" s="9">
-        <f t="shared" si="3"/>
-        <v>0.72204504685633197</v>
-      </c>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="10"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="E7" s="10"/>
@@ -24585,42 +24434,6 @@
       <c r="I19" s="11"/>
       <c r="J19" s="11"/>
       <c r="K19" s="10"/>
-    </row>
-    <row r="20" spans="5:11" x14ac:dyDescent="0.2">
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="10"/>
-    </row>
-    <row r="21" spans="5:11" x14ac:dyDescent="0.2">
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="10"/>
-    </row>
-    <row r="22" spans="5:11" x14ac:dyDescent="0.2">
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="10"/>
-    </row>
-    <row r="23" spans="5:11" x14ac:dyDescent="0.2">
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24658,10 +24471,10 @@
         <v>391</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>395</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>396</v>
       </c>
       <c r="G1" s="1"/>
     </row>
@@ -24693,57 +24506,57 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>398</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>391</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="L5" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>422</v>
-      </c>
       <c r="N5" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="P5" s="1" t="s">
         <v>419</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B6" s="1">
         <v>1</v>
@@ -24752,7 +24565,7 @@
         <v>389</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="E6" s="1">
         <v>0.94499999999999995</v>
@@ -24774,7 +24587,7 @@
         <v>-1.9985536081552357E-2</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K6" s="1">
         <v>-112</v>
@@ -24799,7 +24612,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B7" s="1">
         <f>B6+1</f>
@@ -24809,7 +24622,7 @@
         <v>389</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E7" s="1">
         <v>0.68979999999999997</v>
@@ -24831,7 +24644,7 @@
         <v>-7.3041333591230655E-3</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K7" s="1">
         <v>-103</v>
@@ -24856,7 +24669,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B8" s="1">
         <f t="shared" ref="B8:B16" si="4">B7+1</f>
@@ -24866,7 +24679,7 @@
         <v>388</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="E8" s="1">
         <v>0.74019999999999997</v>
@@ -24888,7 +24701,7 @@
         <v>3.1073790677935476E-2</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K8" s="1">
         <v>-110</v>
@@ -24913,7 +24726,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="B9" s="1">
         <f t="shared" si="4"/>
@@ -24923,7 +24736,7 @@
         <v>388</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E9" s="1">
         <v>0.67900000000000005</v>
@@ -24945,7 +24758,7 @@
         <v>2.5431238755099773E-2</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K9" s="1">
         <v>-110</v>
@@ -24970,7 +24783,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B10" s="1">
         <f t="shared" si="4"/>
@@ -24980,7 +24793,7 @@
         <v>389</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="E10" s="1">
         <v>1.2898000000000001</v>
@@ -25002,7 +24815,7 @@
         <v>1.2346518407494022E-2</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K10" s="1">
         <v>-112</v>
@@ -25027,7 +24840,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B11" s="1">
         <f t="shared" si="4"/>
@@ -25037,7 +24850,7 @@
         <v>389</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="E11" s="1">
         <v>0.68820000000000003</v>
@@ -25059,7 +24872,7 @@
         <v>2.5460169228087515E-2</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K11" s="1">
         <v>-109</v>
@@ -25084,7 +24897,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B12" s="1">
         <f t="shared" si="4"/>
@@ -25094,7 +24907,7 @@
         <v>389</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="E12" s="1">
         <v>0.69510000000000005</v>
@@ -25116,7 +24929,7 @@
         <v>4.1788135989584758E-2</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K12" s="1">
         <v>-109</v>
@@ -25141,7 +24954,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B13" s="1">
         <f t="shared" si="4"/>
@@ -25151,7 +24964,7 @@
         <v>389</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E13" s="1">
         <v>1.0744</v>
@@ -25173,7 +24986,7 @@
         <v>3.4345868990886666E-2</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K13" s="1">
         <v>-107</v>
@@ -25198,7 +25011,7 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B14" s="1">
         <f t="shared" si="4"/>
@@ -25208,7 +25021,7 @@
         <v>388</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E14" s="1">
         <v>1.0632999999999999</v>
@@ -25230,7 +25043,7 @@
         <v>3.3490856499044576E-2</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K14" s="1">
         <v>-110</v>
@@ -25255,7 +25068,7 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B15" s="1">
         <f t="shared" si="4"/>
@@ -25265,7 +25078,7 @@
         <v>389</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="E15" s="1">
         <v>0.82620000000000005</v>
@@ -25287,7 +25100,7 @@
         <v>2.681961318224562E-2</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K15" s="1">
         <v>-109</v>
@@ -25312,7 +25125,7 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B16" s="1">
         <f t="shared" si="4"/>
@@ -25322,7 +25135,7 @@
         <v>388</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E16" s="1">
         <v>0.72199999999999998</v>
@@ -25344,7 +25157,7 @@
         <v>2.4502342779500797E-2</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K16" s="1">
         <v>-110</v>
@@ -25631,45 +25444,45 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>411</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
@@ -25684,10 +25497,10 @@
         <v>475</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="K2" s="1">
         <f>IF(J2="W",(D2/100)*E2,IF(J2="",0,-E2))</f>
@@ -25696,10 +25509,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>30</v>
@@ -25714,10 +25527,10 @@
         <v>6000</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="K3" s="1">
         <f t="shared" ref="K3:K5" si="0">IF(J3="W",(D3/100)*E3,IF(J3="",0,-E3))</f>
@@ -25726,10 +25539,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>13</v>
@@ -25744,10 +25557,10 @@
         <v>1800</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="K4" s="1">
         <f t="shared" si="0"/>
@@ -25756,10 +25569,10 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>48</v>
@@ -25774,10 +25587,10 @@
         <v>50000</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="K5" s="1">
         <f t="shared" si="0"/>
@@ -25808,7 +25621,7 @@
         <v>366</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -33583,7 +33396,7 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B61">
         <v>7.9899999999999999E-2</v>

</xml_diff>

<commit_message>
Update projections show flag
</commit_message>
<xml_diff>
--- a/WebsiteData.xlsx
+++ b/WebsiteData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkevans/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D37BB91C-3606-1347-8863-5D322282D70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CFF2058-DF5C-9F4E-8888-BD775227A124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="27580" windowHeight="20000" xr2:uid="{C762ECBC-EE1A-4249-820F-B10BC232F997}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="16140" windowHeight="20000" xr2:uid="{C762ECBC-EE1A-4249-820F-B10BC232F997}"/>
   </bookViews>
   <sheets>
     <sheet name="Projections" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="445">
   <si>
     <t>Team</t>
   </si>
@@ -1374,6 +1374,12 @@
   </si>
   <si>
     <t>KENN/LT</t>
+  </si>
+  <si>
+    <t>Show</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -24195,7 +24201,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2A118F-D7F3-5348-BECB-A41992F5CAD2}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -24208,7 +24214,7 @@
     <col min="8" max="11" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>373</v>
       </c>
@@ -24242,8 +24248,11 @@
       <c r="K1" s="1" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L1" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="e">
         <f>VLOOKUP(A2,[1]Games!$B$2:$K$398,2,FALSE)</f>
         <v>#N/A</v>
@@ -24281,8 +24290,11 @@
         <f>IF(J2="Yes",(H2*1500)/100,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" s="1" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
       <c r="G3" s="11"/>
@@ -24291,7 +24303,7 @@
       <c r="J3" s="11"/>
       <c r="K3" s="10"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
       <c r="G4" s="11"/>
@@ -24300,7 +24312,7 @@
       <c r="J4" s="11"/>
       <c r="K4" s="10"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
       <c r="G5" s="11"/>
@@ -24309,7 +24321,7 @@
       <c r="J5" s="11"/>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
       <c r="G6" s="11"/>
@@ -24318,7 +24330,7 @@
       <c r="J6" s="11"/>
       <c r="K6" s="10"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="11"/>
@@ -24327,7 +24339,7 @@
       <c r="J7" s="11"/>
       <c r="K7" s="10"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
       <c r="G8" s="11"/>
@@ -24336,7 +24348,7 @@
       <c r="J8" s="11"/>
       <c r="K8" s="10"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
       <c r="G9" s="11"/>
@@ -24345,7 +24357,7 @@
       <c r="J9" s="11"/>
       <c r="K9" s="10"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
       <c r="G10" s="11"/>
@@ -24354,7 +24366,7 @@
       <c r="J10" s="11"/>
       <c r="K10" s="10"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
       <c r="G11" s="11"/>
@@ -24363,7 +24375,7 @@
       <c r="J11" s="11"/>
       <c r="K11" s="10"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
       <c r="G12" s="11"/>
@@ -24372,7 +24384,7 @@
       <c r="J12" s="11"/>
       <c r="K12" s="10"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
       <c r="G13" s="11"/>
@@ -24381,7 +24393,7 @@
       <c r="J13" s="11"/>
       <c r="K13" s="10"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
       <c r="G14" s="11"/>
@@ -24390,7 +24402,7 @@
       <c r="J14" s="11"/>
       <c r="K14" s="10"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="11"/>
@@ -24399,7 +24411,7 @@
       <c r="J15" s="11"/>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
       <c r="G16" s="11"/>

</xml_diff>

<commit_message>
Add odds column to projections
</commit_message>
<xml_diff>
--- a/WebsiteData.xlsx
+++ b/WebsiteData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jkevans/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F47787EA-0E91-5441-8D93-15FECB3664D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE0352D0-A2A8-2343-9AD1-C3E281D15A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19960" xr2:uid="{C762ECBC-EE1A-4249-820F-B10BC232F997}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="20680" windowHeight="19940" xr2:uid="{C762ECBC-EE1A-4249-820F-B10BC232F997}"/>
   </bookViews>
   <sheets>
     <sheet name="Projections" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="465">
   <si>
     <t>Team</t>
   </si>
@@ -1656,7 +1656,7 @@
             <v>5.7780905774790781E-2</v>
           </cell>
           <cell r="J3">
-            <v>0.44652162262184469</v>
+            <v>0.44652162262184492</v>
           </cell>
           <cell r="K3">
             <v>0</v>
@@ -1673,19 +1673,19 @@
             <v>Iowa</v>
           </cell>
           <cell r="E4">
-            <v>5.5829743724806304</v>
+            <v>5.257974372480632</v>
           </cell>
           <cell r="F4" t="b">
             <v>0</v>
           </cell>
           <cell r="G4">
-            <v>0.58859640890923282</v>
+            <v>0.59284650142001671</v>
           </cell>
           <cell r="H4">
             <v>0</v>
           </cell>
           <cell r="I4">
-            <v>0.1236840533721718</v>
+            <v>0.1317978663473047</v>
           </cell>
           <cell r="J4">
             <v>0.38710225177014629</v>
@@ -1769,7 +1769,7 @@
             <v>Tennessee</v>
           </cell>
           <cell r="E7">
-            <v>6.1693961042649601</v>
+            <v>6.1693961042649592</v>
           </cell>
           <cell r="F7" t="b">
             <v>0</v>
@@ -1784,7 +1784,7 @@
             <v>5.7495491589876317E-2</v>
           </cell>
           <cell r="J7">
-            <v>0.32440678103529169</v>
+            <v>0.32440678103529158</v>
           </cell>
           <cell r="K7">
             <v>0</v>
@@ -1929,22 +1929,22 @@
             <v>Nebraska</v>
           </cell>
           <cell r="E12">
-            <v>0.8061527799804542</v>
+            <v>1.131152779980455</v>
           </cell>
           <cell r="F12" t="b">
             <v>0</v>
           </cell>
           <cell r="G12">
-            <v>0.56961125963652415</v>
+            <v>0.5653103859347075</v>
           </cell>
           <cell r="H12">
             <v>0</v>
           </cell>
           <cell r="I12">
-            <v>8.7439677487909817E-2</v>
+            <v>7.9228918602623488E-2</v>
           </cell>
           <cell r="J12">
-            <v>0.19277136123939659</v>
+            <v>0.19277136123939681</v>
           </cell>
           <cell r="K12">
             <v>0</v>
@@ -1993,7 +1993,7 @@
             <v>Duke</v>
           </cell>
           <cell r="E14">
-            <v>-5.7074469950208453</v>
+            <v>-5.7074469950208462</v>
           </cell>
           <cell r="F14" t="b">
             <v>0</v>
@@ -2008,7 +2008,7 @@
             <v>-7.7435986809383786E-3</v>
           </cell>
           <cell r="J14">
-            <v>0.1359058509226507</v>
+            <v>0.13590585092265101</v>
           </cell>
           <cell r="K14">
             <v>0</v>
@@ -2025,7 +2025,7 @@
             <v>Iowa State</v>
           </cell>
           <cell r="E15">
-            <v>0.5490944982080217</v>
+            <v>0.54909449820802081</v>
           </cell>
           <cell r="F15" t="b">
             <v>0</v>
@@ -2040,7 +2040,7 @@
             <v>0.16820481729504341</v>
           </cell>
           <cell r="J15">
-            <v>0.28694196100801311</v>
+            <v>0.28694196100801289</v>
           </cell>
           <cell r="K15">
             <v>0</v>
@@ -8904,7 +8904,7 @@
             <v>0</v>
           </cell>
           <cell r="X4">
-            <v>-2</v>
+            <v>-1.5</v>
           </cell>
         </row>
         <row r="5">
@@ -9496,7 +9496,7 @@
             <v>0</v>
           </cell>
           <cell r="X12">
-            <v>2</v>
+            <v>1.5</v>
           </cell>
         </row>
         <row r="13">
@@ -9868,3778 +9868,6 @@
           <cell r="X17">
             <v>10</v>
           </cell>
-        </row>
-        <row r="18">
-          <cell r="D18"/>
-          <cell r="E18"/>
-          <cell r="F18"/>
-          <cell r="G18"/>
-          <cell r="H18"/>
-          <cell r="I18"/>
-          <cell r="J18"/>
-          <cell r="K18"/>
-          <cell r="L18"/>
-          <cell r="M18"/>
-          <cell r="N18"/>
-          <cell r="O18"/>
-          <cell r="P18"/>
-          <cell r="Q18"/>
-          <cell r="R18"/>
-          <cell r="S18"/>
-          <cell r="T18"/>
-          <cell r="U18"/>
-          <cell r="V18"/>
-          <cell r="W18"/>
-          <cell r="X18"/>
-        </row>
-        <row r="19">
-          <cell r="D19"/>
-          <cell r="E19"/>
-          <cell r="F19"/>
-          <cell r="G19"/>
-          <cell r="H19"/>
-          <cell r="I19"/>
-          <cell r="J19"/>
-          <cell r="K19"/>
-          <cell r="L19"/>
-          <cell r="M19"/>
-          <cell r="N19"/>
-          <cell r="O19"/>
-          <cell r="P19"/>
-          <cell r="Q19"/>
-          <cell r="R19"/>
-          <cell r="S19"/>
-          <cell r="T19"/>
-          <cell r="U19"/>
-          <cell r="V19"/>
-          <cell r="W19"/>
-          <cell r="X19"/>
-        </row>
-        <row r="20">
-          <cell r="D20"/>
-          <cell r="E20"/>
-          <cell r="F20"/>
-          <cell r="G20"/>
-          <cell r="H20"/>
-          <cell r="I20"/>
-          <cell r="J20"/>
-          <cell r="K20"/>
-          <cell r="L20"/>
-          <cell r="M20"/>
-          <cell r="N20"/>
-          <cell r="O20"/>
-          <cell r="P20"/>
-          <cell r="Q20"/>
-          <cell r="R20"/>
-          <cell r="S20"/>
-          <cell r="T20"/>
-          <cell r="U20"/>
-          <cell r="V20"/>
-          <cell r="W20"/>
-          <cell r="X20"/>
-        </row>
-        <row r="21">
-          <cell r="D21"/>
-          <cell r="E21"/>
-          <cell r="F21"/>
-          <cell r="G21"/>
-          <cell r="H21"/>
-          <cell r="I21"/>
-          <cell r="J21"/>
-          <cell r="K21"/>
-          <cell r="L21"/>
-          <cell r="M21"/>
-          <cell r="N21"/>
-          <cell r="O21"/>
-          <cell r="P21"/>
-          <cell r="Q21"/>
-          <cell r="R21"/>
-          <cell r="S21"/>
-          <cell r="T21"/>
-          <cell r="U21"/>
-          <cell r="V21"/>
-          <cell r="W21"/>
-          <cell r="X21"/>
-        </row>
-        <row r="22">
-          <cell r="D22"/>
-          <cell r="E22"/>
-          <cell r="F22"/>
-          <cell r="G22"/>
-          <cell r="H22"/>
-          <cell r="I22"/>
-          <cell r="J22"/>
-          <cell r="K22"/>
-          <cell r="L22"/>
-          <cell r="M22"/>
-          <cell r="N22"/>
-          <cell r="O22"/>
-          <cell r="P22"/>
-          <cell r="Q22"/>
-          <cell r="R22"/>
-          <cell r="S22"/>
-          <cell r="T22"/>
-          <cell r="U22"/>
-          <cell r="V22"/>
-          <cell r="W22"/>
-          <cell r="X22"/>
-        </row>
-        <row r="23">
-          <cell r="D23"/>
-          <cell r="E23"/>
-          <cell r="F23"/>
-          <cell r="G23"/>
-          <cell r="H23"/>
-          <cell r="I23"/>
-          <cell r="J23"/>
-          <cell r="K23"/>
-          <cell r="L23"/>
-          <cell r="M23"/>
-          <cell r="N23"/>
-          <cell r="O23"/>
-          <cell r="P23"/>
-          <cell r="Q23"/>
-          <cell r="R23"/>
-          <cell r="S23"/>
-          <cell r="T23"/>
-          <cell r="U23"/>
-          <cell r="V23"/>
-          <cell r="W23"/>
-          <cell r="X23"/>
-        </row>
-        <row r="24">
-          <cell r="D24"/>
-          <cell r="E24"/>
-          <cell r="F24"/>
-          <cell r="G24"/>
-          <cell r="H24"/>
-          <cell r="I24"/>
-          <cell r="J24"/>
-          <cell r="K24"/>
-          <cell r="L24"/>
-          <cell r="M24"/>
-          <cell r="N24"/>
-          <cell r="O24"/>
-          <cell r="P24"/>
-          <cell r="Q24"/>
-          <cell r="R24"/>
-          <cell r="S24"/>
-          <cell r="T24"/>
-          <cell r="U24"/>
-          <cell r="V24"/>
-          <cell r="W24"/>
-          <cell r="X24"/>
-        </row>
-        <row r="25">
-          <cell r="D25"/>
-          <cell r="E25"/>
-          <cell r="F25"/>
-          <cell r="G25"/>
-          <cell r="H25"/>
-          <cell r="I25"/>
-          <cell r="J25"/>
-          <cell r="K25"/>
-          <cell r="L25"/>
-          <cell r="M25"/>
-          <cell r="N25"/>
-          <cell r="O25"/>
-          <cell r="P25"/>
-          <cell r="Q25"/>
-          <cell r="R25"/>
-          <cell r="S25"/>
-          <cell r="T25"/>
-          <cell r="U25"/>
-          <cell r="V25"/>
-          <cell r="W25"/>
-          <cell r="X25"/>
-        </row>
-        <row r="26">
-          <cell r="D26"/>
-          <cell r="E26"/>
-          <cell r="F26"/>
-          <cell r="G26"/>
-          <cell r="H26"/>
-          <cell r="I26"/>
-          <cell r="J26"/>
-          <cell r="K26"/>
-          <cell r="L26"/>
-          <cell r="M26"/>
-          <cell r="N26"/>
-          <cell r="O26"/>
-          <cell r="P26"/>
-          <cell r="Q26"/>
-          <cell r="R26"/>
-          <cell r="S26"/>
-          <cell r="T26"/>
-          <cell r="U26"/>
-          <cell r="V26"/>
-          <cell r="W26"/>
-          <cell r="X26"/>
-        </row>
-        <row r="27">
-          <cell r="D27"/>
-          <cell r="E27"/>
-          <cell r="F27"/>
-          <cell r="G27"/>
-          <cell r="H27"/>
-          <cell r="I27"/>
-          <cell r="J27"/>
-          <cell r="K27"/>
-          <cell r="L27"/>
-          <cell r="M27"/>
-          <cell r="N27"/>
-          <cell r="O27"/>
-          <cell r="P27"/>
-          <cell r="Q27"/>
-          <cell r="R27"/>
-          <cell r="S27"/>
-          <cell r="T27"/>
-          <cell r="U27"/>
-          <cell r="V27"/>
-          <cell r="W27"/>
-          <cell r="X27"/>
-        </row>
-        <row r="28">
-          <cell r="D28"/>
-          <cell r="E28"/>
-          <cell r="F28"/>
-          <cell r="G28"/>
-          <cell r="H28"/>
-          <cell r="I28"/>
-          <cell r="J28"/>
-          <cell r="K28"/>
-          <cell r="L28"/>
-          <cell r="M28"/>
-          <cell r="N28"/>
-          <cell r="O28"/>
-          <cell r="P28"/>
-          <cell r="Q28"/>
-          <cell r="R28"/>
-          <cell r="S28"/>
-          <cell r="T28"/>
-          <cell r="U28"/>
-          <cell r="V28"/>
-          <cell r="W28"/>
-          <cell r="X28"/>
-        </row>
-        <row r="29">
-          <cell r="D29"/>
-          <cell r="E29"/>
-          <cell r="F29"/>
-          <cell r="G29"/>
-          <cell r="H29"/>
-          <cell r="I29"/>
-          <cell r="J29"/>
-          <cell r="K29"/>
-          <cell r="L29"/>
-          <cell r="M29"/>
-          <cell r="N29"/>
-          <cell r="O29"/>
-          <cell r="P29"/>
-          <cell r="Q29"/>
-          <cell r="R29"/>
-          <cell r="S29"/>
-          <cell r="T29"/>
-          <cell r="U29"/>
-          <cell r="V29"/>
-          <cell r="W29"/>
-          <cell r="X29"/>
-        </row>
-        <row r="30">
-          <cell r="D30"/>
-          <cell r="E30"/>
-          <cell r="F30"/>
-          <cell r="G30"/>
-          <cell r="H30"/>
-          <cell r="I30"/>
-          <cell r="J30"/>
-          <cell r="K30"/>
-          <cell r="L30"/>
-          <cell r="M30"/>
-          <cell r="N30"/>
-          <cell r="O30"/>
-          <cell r="P30"/>
-          <cell r="Q30"/>
-          <cell r="R30"/>
-          <cell r="S30"/>
-          <cell r="T30"/>
-          <cell r="U30"/>
-          <cell r="V30"/>
-          <cell r="W30"/>
-          <cell r="X30"/>
-        </row>
-        <row r="31">
-          <cell r="D31"/>
-          <cell r="E31"/>
-          <cell r="F31"/>
-          <cell r="G31"/>
-          <cell r="H31"/>
-          <cell r="I31"/>
-          <cell r="J31"/>
-          <cell r="K31"/>
-          <cell r="L31"/>
-          <cell r="M31"/>
-          <cell r="N31"/>
-          <cell r="O31"/>
-          <cell r="P31"/>
-          <cell r="Q31"/>
-          <cell r="R31"/>
-          <cell r="S31"/>
-          <cell r="T31"/>
-          <cell r="U31"/>
-          <cell r="V31"/>
-          <cell r="W31"/>
-          <cell r="X31"/>
-        </row>
-        <row r="32">
-          <cell r="D32"/>
-          <cell r="E32"/>
-          <cell r="F32"/>
-          <cell r="G32"/>
-          <cell r="H32"/>
-          <cell r="I32"/>
-          <cell r="J32"/>
-          <cell r="K32"/>
-          <cell r="L32"/>
-          <cell r="M32"/>
-          <cell r="N32"/>
-          <cell r="O32"/>
-          <cell r="P32"/>
-          <cell r="Q32"/>
-          <cell r="R32"/>
-          <cell r="S32"/>
-          <cell r="T32"/>
-          <cell r="U32"/>
-          <cell r="V32"/>
-          <cell r="W32"/>
-          <cell r="X32"/>
-        </row>
-        <row r="33">
-          <cell r="D33"/>
-          <cell r="E33"/>
-          <cell r="F33"/>
-          <cell r="G33"/>
-          <cell r="H33"/>
-          <cell r="I33"/>
-          <cell r="J33"/>
-          <cell r="K33"/>
-          <cell r="L33"/>
-          <cell r="M33"/>
-          <cell r="N33"/>
-          <cell r="O33"/>
-          <cell r="P33"/>
-          <cell r="Q33"/>
-          <cell r="R33"/>
-          <cell r="S33"/>
-          <cell r="T33"/>
-          <cell r="U33"/>
-          <cell r="V33"/>
-          <cell r="W33"/>
-          <cell r="X33"/>
-        </row>
-        <row r="34">
-          <cell r="D34"/>
-          <cell r="E34"/>
-          <cell r="F34"/>
-          <cell r="G34"/>
-          <cell r="H34"/>
-          <cell r="I34"/>
-          <cell r="J34"/>
-          <cell r="K34"/>
-          <cell r="L34"/>
-          <cell r="M34"/>
-          <cell r="N34"/>
-          <cell r="O34"/>
-          <cell r="P34"/>
-          <cell r="Q34"/>
-          <cell r="R34"/>
-          <cell r="S34"/>
-          <cell r="T34"/>
-          <cell r="U34"/>
-          <cell r="V34"/>
-          <cell r="W34"/>
-          <cell r="X34"/>
-        </row>
-        <row r="35">
-          <cell r="D35"/>
-          <cell r="E35"/>
-          <cell r="F35"/>
-          <cell r="G35"/>
-          <cell r="H35"/>
-          <cell r="I35"/>
-          <cell r="J35"/>
-          <cell r="K35"/>
-          <cell r="L35"/>
-          <cell r="M35"/>
-          <cell r="N35"/>
-          <cell r="O35"/>
-          <cell r="P35"/>
-          <cell r="Q35"/>
-          <cell r="R35"/>
-          <cell r="S35"/>
-          <cell r="T35"/>
-          <cell r="U35"/>
-          <cell r="V35"/>
-          <cell r="W35"/>
-          <cell r="X35"/>
-        </row>
-        <row r="36">
-          <cell r="D36"/>
-          <cell r="E36"/>
-          <cell r="F36"/>
-          <cell r="G36"/>
-          <cell r="H36"/>
-          <cell r="I36"/>
-          <cell r="J36"/>
-          <cell r="K36"/>
-          <cell r="L36"/>
-          <cell r="M36"/>
-          <cell r="N36"/>
-          <cell r="O36"/>
-          <cell r="P36"/>
-          <cell r="Q36"/>
-          <cell r="R36"/>
-          <cell r="S36"/>
-          <cell r="T36"/>
-          <cell r="U36"/>
-          <cell r="V36"/>
-          <cell r="W36"/>
-          <cell r="X36"/>
-        </row>
-        <row r="37">
-          <cell r="D37"/>
-          <cell r="E37"/>
-          <cell r="F37"/>
-          <cell r="G37"/>
-          <cell r="H37"/>
-          <cell r="I37"/>
-          <cell r="J37"/>
-          <cell r="K37"/>
-          <cell r="L37"/>
-          <cell r="M37"/>
-          <cell r="N37"/>
-          <cell r="O37"/>
-          <cell r="P37"/>
-          <cell r="Q37"/>
-          <cell r="R37"/>
-          <cell r="S37"/>
-          <cell r="T37"/>
-          <cell r="U37"/>
-          <cell r="V37"/>
-          <cell r="W37"/>
-          <cell r="X37"/>
-        </row>
-        <row r="38">
-          <cell r="D38"/>
-          <cell r="E38"/>
-          <cell r="F38"/>
-          <cell r="G38"/>
-          <cell r="H38"/>
-          <cell r="I38"/>
-          <cell r="J38"/>
-          <cell r="K38"/>
-          <cell r="L38"/>
-          <cell r="M38"/>
-          <cell r="N38"/>
-          <cell r="O38"/>
-          <cell r="P38"/>
-          <cell r="Q38"/>
-          <cell r="R38"/>
-          <cell r="S38"/>
-          <cell r="T38"/>
-          <cell r="U38"/>
-          <cell r="V38"/>
-          <cell r="W38"/>
-          <cell r="X38"/>
-        </row>
-        <row r="39">
-          <cell r="D39"/>
-          <cell r="E39"/>
-          <cell r="F39"/>
-          <cell r="G39"/>
-          <cell r="H39"/>
-          <cell r="I39"/>
-          <cell r="J39"/>
-          <cell r="K39"/>
-          <cell r="L39"/>
-          <cell r="M39"/>
-          <cell r="N39"/>
-          <cell r="O39"/>
-          <cell r="P39"/>
-          <cell r="Q39"/>
-          <cell r="R39"/>
-          <cell r="S39"/>
-          <cell r="T39"/>
-          <cell r="U39"/>
-          <cell r="V39"/>
-          <cell r="W39"/>
-          <cell r="X39"/>
-        </row>
-        <row r="40">
-          <cell r="D40"/>
-          <cell r="E40"/>
-          <cell r="F40"/>
-          <cell r="G40"/>
-          <cell r="H40"/>
-          <cell r="I40"/>
-          <cell r="J40"/>
-          <cell r="K40"/>
-          <cell r="L40"/>
-          <cell r="M40"/>
-          <cell r="N40"/>
-          <cell r="O40"/>
-          <cell r="P40"/>
-          <cell r="Q40"/>
-          <cell r="R40"/>
-          <cell r="S40"/>
-          <cell r="T40"/>
-          <cell r="U40"/>
-          <cell r="V40"/>
-          <cell r="W40"/>
-          <cell r="X40"/>
-        </row>
-        <row r="41">
-          <cell r="D41"/>
-          <cell r="E41"/>
-          <cell r="F41"/>
-          <cell r="G41"/>
-          <cell r="H41"/>
-          <cell r="I41"/>
-          <cell r="J41"/>
-          <cell r="K41"/>
-          <cell r="L41"/>
-          <cell r="M41"/>
-          <cell r="N41"/>
-          <cell r="O41"/>
-          <cell r="P41"/>
-          <cell r="Q41"/>
-          <cell r="R41"/>
-          <cell r="S41"/>
-          <cell r="T41"/>
-          <cell r="U41"/>
-          <cell r="V41"/>
-          <cell r="W41"/>
-          <cell r="X41"/>
-        </row>
-        <row r="42">
-          <cell r="D42"/>
-          <cell r="E42"/>
-          <cell r="F42"/>
-          <cell r="G42"/>
-          <cell r="H42"/>
-          <cell r="I42"/>
-          <cell r="J42"/>
-          <cell r="K42"/>
-          <cell r="L42"/>
-          <cell r="M42"/>
-          <cell r="N42"/>
-          <cell r="O42"/>
-          <cell r="P42"/>
-          <cell r="Q42"/>
-          <cell r="R42"/>
-          <cell r="S42"/>
-          <cell r="T42"/>
-          <cell r="U42"/>
-          <cell r="V42"/>
-          <cell r="W42"/>
-          <cell r="X42"/>
-        </row>
-        <row r="43">
-          <cell r="D43"/>
-          <cell r="E43"/>
-          <cell r="F43"/>
-          <cell r="G43"/>
-          <cell r="H43"/>
-          <cell r="I43"/>
-          <cell r="J43"/>
-          <cell r="K43"/>
-          <cell r="L43"/>
-          <cell r="M43"/>
-          <cell r="N43"/>
-          <cell r="O43"/>
-          <cell r="P43"/>
-          <cell r="Q43"/>
-          <cell r="R43"/>
-          <cell r="S43"/>
-          <cell r="T43"/>
-          <cell r="U43"/>
-          <cell r="V43"/>
-          <cell r="W43"/>
-          <cell r="X43"/>
-        </row>
-        <row r="44">
-          <cell r="D44"/>
-          <cell r="E44"/>
-          <cell r="F44"/>
-          <cell r="G44"/>
-          <cell r="H44"/>
-          <cell r="I44"/>
-          <cell r="J44"/>
-          <cell r="K44"/>
-          <cell r="L44"/>
-          <cell r="M44"/>
-          <cell r="N44"/>
-          <cell r="O44"/>
-          <cell r="P44"/>
-          <cell r="Q44"/>
-          <cell r="R44"/>
-          <cell r="S44"/>
-          <cell r="T44"/>
-          <cell r="U44"/>
-          <cell r="V44"/>
-          <cell r="W44"/>
-          <cell r="X44"/>
-        </row>
-        <row r="45">
-          <cell r="D45"/>
-          <cell r="E45"/>
-          <cell r="F45"/>
-          <cell r="G45"/>
-          <cell r="H45"/>
-          <cell r="I45"/>
-          <cell r="J45"/>
-          <cell r="K45"/>
-          <cell r="L45"/>
-          <cell r="M45"/>
-          <cell r="N45"/>
-          <cell r="O45"/>
-          <cell r="P45"/>
-          <cell r="Q45"/>
-          <cell r="R45"/>
-          <cell r="S45"/>
-          <cell r="T45"/>
-          <cell r="U45"/>
-          <cell r="V45"/>
-          <cell r="W45"/>
-          <cell r="X45"/>
-        </row>
-        <row r="46">
-          <cell r="D46"/>
-          <cell r="E46"/>
-          <cell r="F46"/>
-          <cell r="G46"/>
-          <cell r="H46"/>
-          <cell r="I46"/>
-          <cell r="J46"/>
-          <cell r="K46"/>
-          <cell r="L46"/>
-          <cell r="M46"/>
-          <cell r="N46"/>
-          <cell r="O46"/>
-          <cell r="P46"/>
-          <cell r="Q46"/>
-          <cell r="R46"/>
-          <cell r="S46"/>
-          <cell r="T46"/>
-          <cell r="U46"/>
-          <cell r="V46"/>
-          <cell r="W46"/>
-          <cell r="X46"/>
-        </row>
-        <row r="47">
-          <cell r="D47"/>
-          <cell r="E47"/>
-          <cell r="F47"/>
-          <cell r="G47"/>
-          <cell r="H47"/>
-          <cell r="I47"/>
-          <cell r="J47"/>
-          <cell r="K47"/>
-          <cell r="L47"/>
-          <cell r="M47"/>
-          <cell r="N47"/>
-          <cell r="O47"/>
-          <cell r="P47"/>
-          <cell r="Q47"/>
-          <cell r="R47"/>
-          <cell r="S47"/>
-          <cell r="T47"/>
-          <cell r="U47"/>
-          <cell r="V47"/>
-          <cell r="W47"/>
-          <cell r="X47"/>
-        </row>
-        <row r="48">
-          <cell r="D48"/>
-          <cell r="E48"/>
-          <cell r="F48"/>
-          <cell r="G48"/>
-          <cell r="H48"/>
-          <cell r="I48"/>
-          <cell r="J48"/>
-          <cell r="K48"/>
-          <cell r="L48"/>
-          <cell r="M48"/>
-          <cell r="N48"/>
-          <cell r="O48"/>
-          <cell r="P48"/>
-          <cell r="Q48"/>
-          <cell r="R48"/>
-          <cell r="S48"/>
-          <cell r="T48"/>
-          <cell r="U48"/>
-          <cell r="V48"/>
-          <cell r="W48"/>
-          <cell r="X48"/>
-        </row>
-        <row r="49">
-          <cell r="D49"/>
-          <cell r="E49"/>
-          <cell r="F49"/>
-          <cell r="G49"/>
-          <cell r="H49"/>
-          <cell r="I49"/>
-          <cell r="J49"/>
-          <cell r="K49"/>
-          <cell r="L49"/>
-          <cell r="M49"/>
-          <cell r="N49"/>
-          <cell r="O49"/>
-          <cell r="P49"/>
-          <cell r="Q49"/>
-          <cell r="R49"/>
-          <cell r="S49"/>
-          <cell r="T49"/>
-          <cell r="U49"/>
-          <cell r="V49"/>
-          <cell r="W49"/>
-          <cell r="X49"/>
-        </row>
-        <row r="50">
-          <cell r="D50"/>
-          <cell r="E50"/>
-          <cell r="F50"/>
-          <cell r="G50"/>
-          <cell r="H50"/>
-          <cell r="I50"/>
-          <cell r="J50"/>
-          <cell r="K50"/>
-          <cell r="L50"/>
-          <cell r="M50"/>
-          <cell r="N50"/>
-          <cell r="O50"/>
-          <cell r="P50"/>
-          <cell r="Q50"/>
-          <cell r="R50"/>
-          <cell r="S50"/>
-          <cell r="T50"/>
-          <cell r="U50"/>
-          <cell r="V50"/>
-          <cell r="W50"/>
-          <cell r="X50"/>
-        </row>
-        <row r="51">
-          <cell r="D51"/>
-          <cell r="E51"/>
-          <cell r="F51"/>
-          <cell r="G51"/>
-          <cell r="H51"/>
-          <cell r="I51"/>
-          <cell r="J51"/>
-          <cell r="K51"/>
-          <cell r="L51"/>
-          <cell r="M51"/>
-          <cell r="N51"/>
-          <cell r="O51"/>
-          <cell r="P51"/>
-          <cell r="Q51"/>
-          <cell r="R51"/>
-          <cell r="S51"/>
-          <cell r="T51"/>
-          <cell r="U51"/>
-          <cell r="V51"/>
-          <cell r="W51"/>
-          <cell r="X51"/>
-        </row>
-        <row r="52">
-          <cell r="D52"/>
-          <cell r="E52"/>
-          <cell r="F52"/>
-          <cell r="G52"/>
-          <cell r="H52"/>
-          <cell r="I52"/>
-          <cell r="J52"/>
-          <cell r="K52"/>
-          <cell r="L52"/>
-          <cell r="M52"/>
-          <cell r="N52"/>
-          <cell r="O52"/>
-          <cell r="P52"/>
-          <cell r="Q52"/>
-          <cell r="R52"/>
-          <cell r="S52"/>
-          <cell r="T52"/>
-          <cell r="U52"/>
-          <cell r="V52"/>
-          <cell r="W52"/>
-          <cell r="X52"/>
-        </row>
-        <row r="53">
-          <cell r="D53"/>
-          <cell r="E53"/>
-          <cell r="F53"/>
-          <cell r="G53"/>
-          <cell r="H53"/>
-          <cell r="I53"/>
-          <cell r="J53"/>
-          <cell r="K53"/>
-          <cell r="L53"/>
-          <cell r="M53"/>
-          <cell r="N53"/>
-          <cell r="O53"/>
-          <cell r="P53"/>
-          <cell r="Q53"/>
-          <cell r="R53"/>
-          <cell r="S53"/>
-          <cell r="T53"/>
-          <cell r="U53"/>
-          <cell r="V53"/>
-          <cell r="W53"/>
-          <cell r="X53"/>
-        </row>
-        <row r="54">
-          <cell r="D54"/>
-          <cell r="E54"/>
-          <cell r="F54"/>
-          <cell r="G54"/>
-          <cell r="H54"/>
-          <cell r="I54"/>
-          <cell r="J54"/>
-          <cell r="K54"/>
-          <cell r="L54"/>
-          <cell r="M54"/>
-          <cell r="N54"/>
-          <cell r="O54"/>
-          <cell r="P54"/>
-          <cell r="Q54"/>
-          <cell r="R54"/>
-          <cell r="S54"/>
-          <cell r="T54"/>
-          <cell r="U54"/>
-          <cell r="V54"/>
-          <cell r="W54"/>
-          <cell r="X54"/>
-        </row>
-        <row r="55">
-          <cell r="D55"/>
-          <cell r="E55"/>
-          <cell r="F55"/>
-          <cell r="G55"/>
-          <cell r="H55"/>
-          <cell r="I55"/>
-          <cell r="J55"/>
-          <cell r="K55"/>
-          <cell r="L55"/>
-          <cell r="M55"/>
-          <cell r="N55"/>
-          <cell r="O55"/>
-          <cell r="P55"/>
-          <cell r="Q55"/>
-          <cell r="R55"/>
-          <cell r="S55"/>
-          <cell r="T55"/>
-          <cell r="U55"/>
-          <cell r="V55"/>
-          <cell r="W55"/>
-          <cell r="X55"/>
-        </row>
-        <row r="56">
-          <cell r="D56"/>
-          <cell r="E56"/>
-          <cell r="F56"/>
-          <cell r="G56"/>
-          <cell r="H56"/>
-          <cell r="I56"/>
-          <cell r="J56"/>
-          <cell r="K56"/>
-          <cell r="L56"/>
-          <cell r="M56"/>
-          <cell r="N56"/>
-          <cell r="O56"/>
-          <cell r="P56"/>
-          <cell r="Q56"/>
-          <cell r="R56"/>
-          <cell r="S56"/>
-          <cell r="T56"/>
-          <cell r="U56"/>
-          <cell r="V56"/>
-          <cell r="W56"/>
-          <cell r="X56"/>
-        </row>
-        <row r="57">
-          <cell r="D57"/>
-          <cell r="E57"/>
-          <cell r="F57"/>
-          <cell r="G57"/>
-          <cell r="H57"/>
-          <cell r="I57"/>
-          <cell r="J57"/>
-          <cell r="K57"/>
-          <cell r="L57"/>
-          <cell r="M57"/>
-          <cell r="N57"/>
-          <cell r="O57"/>
-          <cell r="P57"/>
-          <cell r="Q57"/>
-          <cell r="R57"/>
-          <cell r="S57"/>
-          <cell r="T57"/>
-          <cell r="U57"/>
-          <cell r="V57"/>
-          <cell r="W57"/>
-          <cell r="X57"/>
-        </row>
-        <row r="58">
-          <cell r="D58"/>
-          <cell r="E58"/>
-          <cell r="F58"/>
-          <cell r="G58"/>
-          <cell r="H58"/>
-          <cell r="I58"/>
-          <cell r="J58"/>
-          <cell r="K58"/>
-          <cell r="L58"/>
-          <cell r="M58"/>
-          <cell r="N58"/>
-          <cell r="O58"/>
-          <cell r="P58"/>
-          <cell r="Q58"/>
-          <cell r="R58"/>
-          <cell r="S58"/>
-          <cell r="T58"/>
-          <cell r="U58"/>
-          <cell r="V58"/>
-          <cell r="W58"/>
-          <cell r="X58"/>
-        </row>
-        <row r="59">
-          <cell r="D59"/>
-          <cell r="E59"/>
-          <cell r="F59"/>
-          <cell r="G59"/>
-          <cell r="H59"/>
-          <cell r="I59"/>
-          <cell r="J59"/>
-          <cell r="K59"/>
-          <cell r="L59"/>
-          <cell r="M59"/>
-          <cell r="N59"/>
-          <cell r="O59"/>
-          <cell r="P59"/>
-          <cell r="Q59"/>
-          <cell r="R59"/>
-          <cell r="S59"/>
-          <cell r="T59"/>
-          <cell r="U59"/>
-          <cell r="V59"/>
-          <cell r="W59"/>
-          <cell r="X59"/>
-        </row>
-        <row r="60">
-          <cell r="D60"/>
-          <cell r="E60"/>
-          <cell r="F60"/>
-          <cell r="G60"/>
-          <cell r="H60"/>
-          <cell r="I60"/>
-          <cell r="J60"/>
-          <cell r="K60"/>
-          <cell r="L60"/>
-          <cell r="M60"/>
-          <cell r="N60"/>
-          <cell r="O60"/>
-          <cell r="P60"/>
-          <cell r="Q60"/>
-          <cell r="R60"/>
-          <cell r="S60"/>
-          <cell r="T60"/>
-          <cell r="U60"/>
-          <cell r="V60"/>
-          <cell r="W60"/>
-          <cell r="X60"/>
-        </row>
-        <row r="61">
-          <cell r="D61"/>
-          <cell r="E61"/>
-          <cell r="F61"/>
-          <cell r="G61"/>
-          <cell r="H61"/>
-          <cell r="I61"/>
-          <cell r="J61"/>
-          <cell r="K61"/>
-          <cell r="L61"/>
-          <cell r="M61"/>
-          <cell r="N61"/>
-          <cell r="O61"/>
-          <cell r="P61"/>
-          <cell r="Q61"/>
-          <cell r="R61"/>
-          <cell r="S61"/>
-          <cell r="T61"/>
-          <cell r="U61"/>
-          <cell r="V61"/>
-          <cell r="W61"/>
-          <cell r="X61"/>
-        </row>
-        <row r="62">
-          <cell r="D62"/>
-          <cell r="E62"/>
-          <cell r="F62"/>
-          <cell r="G62"/>
-          <cell r="H62"/>
-          <cell r="I62"/>
-          <cell r="J62"/>
-          <cell r="K62"/>
-          <cell r="L62"/>
-          <cell r="M62"/>
-          <cell r="N62"/>
-          <cell r="O62"/>
-          <cell r="P62"/>
-          <cell r="Q62"/>
-          <cell r="R62"/>
-          <cell r="S62"/>
-          <cell r="T62"/>
-          <cell r="U62"/>
-          <cell r="V62"/>
-          <cell r="W62"/>
-          <cell r="X62"/>
-        </row>
-        <row r="63">
-          <cell r="D63"/>
-          <cell r="E63"/>
-          <cell r="F63"/>
-          <cell r="G63"/>
-          <cell r="H63"/>
-          <cell r="I63"/>
-          <cell r="J63"/>
-          <cell r="K63"/>
-          <cell r="L63"/>
-          <cell r="M63"/>
-          <cell r="N63"/>
-          <cell r="O63"/>
-          <cell r="P63"/>
-          <cell r="Q63"/>
-          <cell r="R63"/>
-          <cell r="S63"/>
-          <cell r="T63"/>
-          <cell r="U63"/>
-          <cell r="V63"/>
-          <cell r="W63"/>
-          <cell r="X63"/>
-        </row>
-        <row r="64">
-          <cell r="D64"/>
-          <cell r="E64"/>
-          <cell r="F64"/>
-          <cell r="G64"/>
-          <cell r="H64"/>
-          <cell r="I64"/>
-          <cell r="J64"/>
-          <cell r="K64"/>
-          <cell r="L64"/>
-          <cell r="M64"/>
-          <cell r="N64"/>
-          <cell r="O64"/>
-          <cell r="P64"/>
-          <cell r="Q64"/>
-          <cell r="R64"/>
-          <cell r="S64"/>
-          <cell r="T64"/>
-          <cell r="U64"/>
-          <cell r="V64"/>
-          <cell r="W64"/>
-          <cell r="X64"/>
-        </row>
-        <row r="65">
-          <cell r="D65"/>
-          <cell r="E65"/>
-          <cell r="F65"/>
-          <cell r="G65"/>
-          <cell r="H65"/>
-          <cell r="I65"/>
-          <cell r="J65"/>
-          <cell r="K65"/>
-          <cell r="L65"/>
-          <cell r="M65"/>
-          <cell r="N65"/>
-          <cell r="O65"/>
-          <cell r="P65"/>
-          <cell r="Q65"/>
-          <cell r="R65"/>
-          <cell r="S65"/>
-          <cell r="T65"/>
-          <cell r="U65"/>
-          <cell r="V65"/>
-          <cell r="W65"/>
-          <cell r="X65"/>
-        </row>
-        <row r="66">
-          <cell r="D66"/>
-          <cell r="E66"/>
-          <cell r="F66"/>
-          <cell r="G66"/>
-          <cell r="H66"/>
-          <cell r="I66"/>
-          <cell r="J66"/>
-          <cell r="K66"/>
-          <cell r="L66"/>
-          <cell r="M66"/>
-          <cell r="N66"/>
-          <cell r="O66"/>
-          <cell r="P66"/>
-          <cell r="Q66"/>
-          <cell r="R66"/>
-          <cell r="S66"/>
-          <cell r="T66"/>
-          <cell r="U66"/>
-          <cell r="V66"/>
-          <cell r="W66"/>
-          <cell r="X66"/>
-        </row>
-        <row r="67">
-          <cell r="D67"/>
-          <cell r="E67"/>
-          <cell r="F67"/>
-          <cell r="G67"/>
-          <cell r="H67"/>
-          <cell r="I67"/>
-          <cell r="J67"/>
-          <cell r="K67"/>
-          <cell r="L67"/>
-          <cell r="M67"/>
-          <cell r="N67"/>
-          <cell r="O67"/>
-          <cell r="P67"/>
-          <cell r="Q67"/>
-          <cell r="R67"/>
-          <cell r="S67"/>
-          <cell r="T67"/>
-          <cell r="U67"/>
-          <cell r="V67"/>
-          <cell r="W67"/>
-          <cell r="X67"/>
-        </row>
-        <row r="68">
-          <cell r="D68"/>
-          <cell r="E68"/>
-          <cell r="F68"/>
-          <cell r="G68"/>
-          <cell r="H68"/>
-          <cell r="I68"/>
-          <cell r="J68"/>
-          <cell r="K68"/>
-          <cell r="L68"/>
-          <cell r="M68"/>
-          <cell r="N68"/>
-          <cell r="O68"/>
-          <cell r="P68"/>
-          <cell r="Q68"/>
-          <cell r="R68"/>
-          <cell r="S68"/>
-          <cell r="T68"/>
-          <cell r="U68"/>
-          <cell r="V68"/>
-          <cell r="W68"/>
-          <cell r="X68"/>
-        </row>
-        <row r="69">
-          <cell r="D69"/>
-          <cell r="E69"/>
-          <cell r="F69"/>
-          <cell r="G69"/>
-          <cell r="H69"/>
-          <cell r="I69"/>
-          <cell r="J69"/>
-          <cell r="K69"/>
-          <cell r="L69"/>
-          <cell r="M69"/>
-          <cell r="N69"/>
-          <cell r="O69"/>
-          <cell r="P69"/>
-          <cell r="Q69"/>
-          <cell r="R69"/>
-          <cell r="S69"/>
-          <cell r="T69"/>
-          <cell r="U69"/>
-          <cell r="V69"/>
-          <cell r="W69"/>
-          <cell r="X69"/>
-        </row>
-        <row r="70">
-          <cell r="D70"/>
-          <cell r="E70"/>
-          <cell r="F70"/>
-          <cell r="G70"/>
-          <cell r="H70"/>
-          <cell r="I70"/>
-          <cell r="J70"/>
-          <cell r="K70"/>
-          <cell r="L70"/>
-          <cell r="M70"/>
-          <cell r="N70"/>
-          <cell r="O70"/>
-          <cell r="P70"/>
-          <cell r="Q70"/>
-          <cell r="R70"/>
-          <cell r="S70"/>
-          <cell r="T70"/>
-          <cell r="U70"/>
-          <cell r="V70"/>
-          <cell r="W70"/>
-          <cell r="X70"/>
-        </row>
-        <row r="71">
-          <cell r="D71"/>
-          <cell r="E71"/>
-          <cell r="F71"/>
-          <cell r="G71"/>
-          <cell r="H71"/>
-          <cell r="I71"/>
-          <cell r="J71"/>
-          <cell r="K71"/>
-          <cell r="L71"/>
-          <cell r="M71"/>
-          <cell r="N71"/>
-          <cell r="O71"/>
-          <cell r="P71"/>
-          <cell r="Q71"/>
-          <cell r="R71"/>
-          <cell r="S71"/>
-          <cell r="T71"/>
-          <cell r="U71"/>
-          <cell r="V71"/>
-          <cell r="W71"/>
-          <cell r="X71"/>
-        </row>
-        <row r="72">
-          <cell r="D72"/>
-          <cell r="E72"/>
-          <cell r="F72"/>
-          <cell r="G72"/>
-          <cell r="H72"/>
-          <cell r="I72"/>
-          <cell r="J72"/>
-          <cell r="K72"/>
-          <cell r="L72"/>
-          <cell r="M72"/>
-          <cell r="N72"/>
-          <cell r="O72"/>
-          <cell r="P72"/>
-          <cell r="Q72"/>
-          <cell r="R72"/>
-          <cell r="S72"/>
-          <cell r="T72"/>
-          <cell r="U72"/>
-          <cell r="V72"/>
-          <cell r="W72"/>
-          <cell r="X72"/>
-        </row>
-        <row r="73">
-          <cell r="D73"/>
-          <cell r="E73"/>
-          <cell r="F73"/>
-          <cell r="G73"/>
-          <cell r="H73"/>
-          <cell r="I73"/>
-          <cell r="J73"/>
-          <cell r="K73"/>
-          <cell r="L73"/>
-          <cell r="M73"/>
-          <cell r="N73"/>
-          <cell r="O73"/>
-          <cell r="P73"/>
-          <cell r="Q73"/>
-          <cell r="R73"/>
-          <cell r="S73"/>
-          <cell r="T73"/>
-          <cell r="U73"/>
-          <cell r="V73"/>
-          <cell r="W73"/>
-          <cell r="X73"/>
-        </row>
-        <row r="74">
-          <cell r="D74"/>
-          <cell r="E74"/>
-          <cell r="F74"/>
-          <cell r="G74"/>
-          <cell r="H74"/>
-          <cell r="I74"/>
-          <cell r="J74"/>
-          <cell r="K74"/>
-          <cell r="L74"/>
-          <cell r="M74"/>
-          <cell r="N74"/>
-          <cell r="O74"/>
-          <cell r="P74"/>
-          <cell r="Q74"/>
-          <cell r="R74"/>
-          <cell r="S74"/>
-          <cell r="T74"/>
-          <cell r="U74"/>
-          <cell r="V74"/>
-          <cell r="W74"/>
-          <cell r="X74"/>
-        </row>
-        <row r="75">
-          <cell r="D75"/>
-          <cell r="E75"/>
-          <cell r="F75"/>
-          <cell r="G75"/>
-          <cell r="H75"/>
-          <cell r="I75"/>
-          <cell r="J75"/>
-          <cell r="K75"/>
-          <cell r="L75"/>
-          <cell r="M75"/>
-          <cell r="N75"/>
-          <cell r="O75"/>
-          <cell r="P75"/>
-          <cell r="Q75"/>
-          <cell r="R75"/>
-          <cell r="S75"/>
-          <cell r="T75"/>
-          <cell r="U75"/>
-          <cell r="V75"/>
-          <cell r="W75"/>
-          <cell r="X75"/>
-        </row>
-        <row r="76">
-          <cell r="D76"/>
-          <cell r="E76"/>
-          <cell r="F76"/>
-          <cell r="G76"/>
-          <cell r="H76"/>
-          <cell r="I76"/>
-          <cell r="J76"/>
-          <cell r="K76"/>
-          <cell r="L76"/>
-          <cell r="M76"/>
-          <cell r="N76"/>
-          <cell r="O76"/>
-          <cell r="P76"/>
-          <cell r="Q76"/>
-          <cell r="R76"/>
-          <cell r="S76"/>
-          <cell r="T76"/>
-          <cell r="U76"/>
-          <cell r="V76"/>
-          <cell r="W76"/>
-          <cell r="X76"/>
-        </row>
-        <row r="77">
-          <cell r="D77"/>
-          <cell r="E77"/>
-          <cell r="F77"/>
-          <cell r="G77"/>
-          <cell r="H77"/>
-          <cell r="I77"/>
-          <cell r="J77"/>
-          <cell r="K77"/>
-          <cell r="L77"/>
-          <cell r="M77"/>
-          <cell r="N77"/>
-          <cell r="O77"/>
-          <cell r="P77"/>
-          <cell r="Q77"/>
-          <cell r="R77"/>
-          <cell r="S77"/>
-          <cell r="T77"/>
-          <cell r="U77"/>
-          <cell r="V77"/>
-          <cell r="W77"/>
-          <cell r="X77"/>
-        </row>
-        <row r="78">
-          <cell r="D78"/>
-          <cell r="E78"/>
-          <cell r="F78"/>
-          <cell r="G78"/>
-          <cell r="H78"/>
-          <cell r="I78"/>
-          <cell r="J78"/>
-          <cell r="K78"/>
-          <cell r="L78"/>
-          <cell r="M78"/>
-          <cell r="N78"/>
-          <cell r="O78"/>
-          <cell r="P78"/>
-          <cell r="Q78"/>
-          <cell r="R78"/>
-          <cell r="S78"/>
-          <cell r="T78"/>
-          <cell r="U78"/>
-          <cell r="V78"/>
-          <cell r="W78"/>
-          <cell r="X78"/>
-        </row>
-        <row r="79">
-          <cell r="D79"/>
-          <cell r="E79"/>
-          <cell r="F79"/>
-          <cell r="G79"/>
-          <cell r="H79"/>
-          <cell r="I79"/>
-          <cell r="J79"/>
-          <cell r="K79"/>
-          <cell r="L79"/>
-          <cell r="M79"/>
-          <cell r="N79"/>
-          <cell r="O79"/>
-          <cell r="P79"/>
-          <cell r="Q79"/>
-          <cell r="R79"/>
-          <cell r="S79"/>
-          <cell r="T79"/>
-          <cell r="U79"/>
-          <cell r="V79"/>
-          <cell r="W79"/>
-          <cell r="X79"/>
-        </row>
-        <row r="80">
-          <cell r="D80"/>
-          <cell r="E80"/>
-          <cell r="F80"/>
-          <cell r="G80"/>
-          <cell r="H80"/>
-          <cell r="I80"/>
-          <cell r="J80"/>
-          <cell r="K80"/>
-          <cell r="L80"/>
-          <cell r="M80"/>
-          <cell r="N80"/>
-          <cell r="O80"/>
-          <cell r="P80"/>
-          <cell r="Q80"/>
-          <cell r="R80"/>
-          <cell r="S80"/>
-          <cell r="T80"/>
-          <cell r="U80"/>
-          <cell r="V80"/>
-          <cell r="W80"/>
-          <cell r="X80"/>
-        </row>
-        <row r="81">
-          <cell r="D81"/>
-          <cell r="E81"/>
-          <cell r="F81"/>
-          <cell r="G81"/>
-          <cell r="H81"/>
-          <cell r="I81"/>
-          <cell r="J81"/>
-          <cell r="K81"/>
-          <cell r="L81"/>
-          <cell r="M81"/>
-          <cell r="N81"/>
-          <cell r="O81"/>
-          <cell r="P81"/>
-          <cell r="Q81"/>
-          <cell r="R81"/>
-          <cell r="S81"/>
-          <cell r="T81"/>
-          <cell r="U81"/>
-          <cell r="V81"/>
-          <cell r="W81"/>
-          <cell r="X81"/>
-        </row>
-        <row r="82">
-          <cell r="D82"/>
-          <cell r="E82"/>
-          <cell r="F82"/>
-          <cell r="G82"/>
-          <cell r="H82"/>
-          <cell r="I82"/>
-          <cell r="J82"/>
-          <cell r="K82"/>
-          <cell r="L82"/>
-          <cell r="M82"/>
-          <cell r="N82"/>
-          <cell r="O82"/>
-          <cell r="P82"/>
-          <cell r="Q82"/>
-          <cell r="R82"/>
-          <cell r="S82"/>
-          <cell r="T82"/>
-          <cell r="U82"/>
-          <cell r="V82"/>
-          <cell r="W82"/>
-          <cell r="X82"/>
-        </row>
-        <row r="83">
-          <cell r="D83"/>
-          <cell r="E83"/>
-          <cell r="F83"/>
-          <cell r="G83"/>
-          <cell r="H83"/>
-          <cell r="I83"/>
-          <cell r="J83"/>
-          <cell r="K83"/>
-          <cell r="L83"/>
-          <cell r="M83"/>
-          <cell r="N83"/>
-          <cell r="O83"/>
-          <cell r="P83"/>
-          <cell r="Q83"/>
-          <cell r="R83"/>
-          <cell r="S83"/>
-          <cell r="T83"/>
-          <cell r="U83"/>
-          <cell r="V83"/>
-          <cell r="W83"/>
-          <cell r="X83"/>
-        </row>
-        <row r="84">
-          <cell r="D84"/>
-          <cell r="E84"/>
-          <cell r="F84"/>
-          <cell r="G84"/>
-          <cell r="H84"/>
-          <cell r="I84"/>
-          <cell r="J84"/>
-          <cell r="K84"/>
-          <cell r="L84"/>
-          <cell r="M84"/>
-          <cell r="N84"/>
-          <cell r="O84"/>
-          <cell r="P84"/>
-          <cell r="Q84"/>
-          <cell r="R84"/>
-          <cell r="S84"/>
-          <cell r="T84"/>
-          <cell r="U84"/>
-          <cell r="V84"/>
-          <cell r="W84"/>
-          <cell r="X84"/>
-        </row>
-        <row r="85">
-          <cell r="D85"/>
-          <cell r="E85"/>
-          <cell r="F85"/>
-          <cell r="G85"/>
-          <cell r="H85"/>
-          <cell r="I85"/>
-          <cell r="J85"/>
-          <cell r="K85"/>
-          <cell r="L85"/>
-          <cell r="M85"/>
-          <cell r="N85"/>
-          <cell r="O85"/>
-          <cell r="P85"/>
-          <cell r="Q85"/>
-          <cell r="R85"/>
-          <cell r="S85"/>
-          <cell r="T85"/>
-          <cell r="U85"/>
-          <cell r="V85"/>
-          <cell r="W85"/>
-          <cell r="X85"/>
-        </row>
-        <row r="86">
-          <cell r="D86"/>
-          <cell r="E86"/>
-          <cell r="F86"/>
-          <cell r="G86"/>
-          <cell r="H86"/>
-          <cell r="I86"/>
-          <cell r="J86"/>
-          <cell r="K86"/>
-          <cell r="L86"/>
-          <cell r="M86"/>
-          <cell r="N86"/>
-          <cell r="O86"/>
-          <cell r="P86"/>
-          <cell r="Q86"/>
-          <cell r="R86"/>
-          <cell r="S86"/>
-          <cell r="T86"/>
-          <cell r="U86"/>
-          <cell r="V86"/>
-          <cell r="W86"/>
-          <cell r="X86"/>
-        </row>
-        <row r="87">
-          <cell r="D87"/>
-          <cell r="E87"/>
-          <cell r="F87"/>
-          <cell r="G87"/>
-          <cell r="H87"/>
-          <cell r="I87"/>
-          <cell r="J87"/>
-          <cell r="K87"/>
-          <cell r="L87"/>
-          <cell r="M87"/>
-          <cell r="N87"/>
-          <cell r="O87"/>
-          <cell r="P87"/>
-          <cell r="Q87"/>
-          <cell r="R87"/>
-          <cell r="S87"/>
-          <cell r="T87"/>
-          <cell r="U87"/>
-          <cell r="V87"/>
-          <cell r="W87"/>
-          <cell r="X87"/>
-        </row>
-        <row r="88">
-          <cell r="D88"/>
-          <cell r="E88"/>
-          <cell r="F88"/>
-          <cell r="G88"/>
-          <cell r="H88"/>
-          <cell r="I88"/>
-          <cell r="J88"/>
-          <cell r="K88"/>
-          <cell r="L88"/>
-          <cell r="M88"/>
-          <cell r="N88"/>
-          <cell r="O88"/>
-          <cell r="P88"/>
-          <cell r="Q88"/>
-          <cell r="R88"/>
-          <cell r="S88"/>
-          <cell r="T88"/>
-          <cell r="U88"/>
-          <cell r="V88"/>
-          <cell r="W88"/>
-          <cell r="X88"/>
-        </row>
-        <row r="89">
-          <cell r="D89"/>
-          <cell r="E89"/>
-          <cell r="F89"/>
-          <cell r="G89"/>
-          <cell r="H89"/>
-          <cell r="I89"/>
-          <cell r="J89"/>
-          <cell r="K89"/>
-          <cell r="L89"/>
-          <cell r="M89"/>
-          <cell r="N89"/>
-          <cell r="O89"/>
-          <cell r="P89"/>
-          <cell r="Q89"/>
-          <cell r="R89"/>
-          <cell r="S89"/>
-          <cell r="T89"/>
-          <cell r="U89"/>
-          <cell r="V89"/>
-          <cell r="W89"/>
-          <cell r="X89"/>
-        </row>
-        <row r="90">
-          <cell r="D90"/>
-          <cell r="E90"/>
-          <cell r="F90"/>
-          <cell r="G90"/>
-          <cell r="H90"/>
-          <cell r="I90"/>
-          <cell r="J90"/>
-          <cell r="K90"/>
-          <cell r="L90"/>
-          <cell r="M90"/>
-          <cell r="N90"/>
-          <cell r="O90"/>
-          <cell r="P90"/>
-          <cell r="Q90"/>
-          <cell r="R90"/>
-          <cell r="S90"/>
-          <cell r="T90"/>
-          <cell r="U90"/>
-          <cell r="V90"/>
-          <cell r="W90"/>
-          <cell r="X90"/>
-        </row>
-        <row r="91">
-          <cell r="D91"/>
-          <cell r="E91"/>
-          <cell r="F91"/>
-          <cell r="G91"/>
-          <cell r="H91"/>
-          <cell r="I91"/>
-          <cell r="J91"/>
-          <cell r="K91"/>
-          <cell r="L91"/>
-          <cell r="M91"/>
-          <cell r="N91"/>
-          <cell r="O91"/>
-          <cell r="P91"/>
-          <cell r="Q91"/>
-          <cell r="R91"/>
-          <cell r="S91"/>
-          <cell r="T91"/>
-          <cell r="U91"/>
-          <cell r="V91"/>
-          <cell r="W91"/>
-          <cell r="X91"/>
-        </row>
-        <row r="92">
-          <cell r="D92"/>
-          <cell r="E92"/>
-          <cell r="F92"/>
-          <cell r="G92"/>
-          <cell r="H92"/>
-          <cell r="I92"/>
-          <cell r="J92"/>
-          <cell r="K92"/>
-          <cell r="L92"/>
-          <cell r="M92"/>
-          <cell r="N92"/>
-          <cell r="O92"/>
-          <cell r="P92"/>
-          <cell r="Q92"/>
-          <cell r="R92"/>
-          <cell r="S92"/>
-          <cell r="T92"/>
-          <cell r="U92"/>
-          <cell r="V92"/>
-          <cell r="W92"/>
-          <cell r="X92"/>
-        </row>
-        <row r="93">
-          <cell r="D93"/>
-          <cell r="E93"/>
-          <cell r="F93"/>
-          <cell r="G93"/>
-          <cell r="H93"/>
-          <cell r="I93"/>
-          <cell r="J93"/>
-          <cell r="K93"/>
-          <cell r="L93"/>
-          <cell r="M93"/>
-          <cell r="N93"/>
-          <cell r="O93"/>
-          <cell r="P93"/>
-          <cell r="Q93"/>
-          <cell r="R93"/>
-          <cell r="S93"/>
-          <cell r="T93"/>
-          <cell r="U93"/>
-          <cell r="V93"/>
-          <cell r="W93"/>
-          <cell r="X93"/>
-        </row>
-        <row r="94">
-          <cell r="D94"/>
-          <cell r="E94"/>
-          <cell r="F94"/>
-          <cell r="G94"/>
-          <cell r="H94"/>
-          <cell r="I94"/>
-          <cell r="J94"/>
-          <cell r="K94"/>
-          <cell r="L94"/>
-          <cell r="M94"/>
-          <cell r="N94"/>
-          <cell r="O94"/>
-          <cell r="P94"/>
-          <cell r="Q94"/>
-          <cell r="R94"/>
-          <cell r="S94"/>
-          <cell r="T94"/>
-          <cell r="U94"/>
-          <cell r="V94"/>
-          <cell r="W94"/>
-          <cell r="X94"/>
-        </row>
-        <row r="95">
-          <cell r="D95"/>
-          <cell r="E95"/>
-          <cell r="F95"/>
-          <cell r="G95"/>
-          <cell r="H95"/>
-          <cell r="I95"/>
-          <cell r="J95"/>
-          <cell r="K95"/>
-          <cell r="L95"/>
-          <cell r="M95"/>
-          <cell r="N95"/>
-          <cell r="O95"/>
-          <cell r="P95"/>
-          <cell r="Q95"/>
-          <cell r="R95"/>
-          <cell r="S95"/>
-          <cell r="T95"/>
-          <cell r="U95"/>
-          <cell r="V95"/>
-          <cell r="W95"/>
-          <cell r="X95"/>
-        </row>
-        <row r="96">
-          <cell r="D96"/>
-          <cell r="E96"/>
-          <cell r="F96"/>
-          <cell r="G96"/>
-          <cell r="H96"/>
-          <cell r="I96"/>
-          <cell r="J96"/>
-          <cell r="K96"/>
-          <cell r="L96"/>
-          <cell r="M96"/>
-          <cell r="N96"/>
-          <cell r="O96"/>
-          <cell r="P96"/>
-          <cell r="Q96"/>
-          <cell r="R96"/>
-          <cell r="S96"/>
-          <cell r="T96"/>
-          <cell r="U96"/>
-          <cell r="V96"/>
-          <cell r="W96"/>
-          <cell r="X96"/>
-        </row>
-        <row r="97">
-          <cell r="D97"/>
-          <cell r="E97"/>
-          <cell r="F97"/>
-          <cell r="G97"/>
-          <cell r="H97"/>
-          <cell r="I97"/>
-          <cell r="J97"/>
-          <cell r="K97"/>
-          <cell r="L97"/>
-          <cell r="M97"/>
-          <cell r="N97"/>
-          <cell r="O97"/>
-          <cell r="P97"/>
-          <cell r="Q97"/>
-          <cell r="R97"/>
-          <cell r="S97"/>
-          <cell r="T97"/>
-          <cell r="U97"/>
-          <cell r="V97"/>
-          <cell r="W97"/>
-          <cell r="X97"/>
-        </row>
-        <row r="98">
-          <cell r="D98"/>
-          <cell r="E98"/>
-          <cell r="F98"/>
-          <cell r="G98"/>
-          <cell r="H98"/>
-          <cell r="I98"/>
-          <cell r="J98"/>
-          <cell r="K98"/>
-          <cell r="L98"/>
-          <cell r="M98"/>
-          <cell r="N98"/>
-          <cell r="O98"/>
-          <cell r="P98"/>
-          <cell r="Q98"/>
-          <cell r="R98"/>
-          <cell r="S98"/>
-          <cell r="T98"/>
-          <cell r="U98"/>
-          <cell r="V98"/>
-          <cell r="W98"/>
-          <cell r="X98"/>
-        </row>
-        <row r="99">
-          <cell r="D99"/>
-          <cell r="E99"/>
-          <cell r="F99"/>
-          <cell r="G99"/>
-          <cell r="H99"/>
-          <cell r="I99"/>
-          <cell r="J99"/>
-          <cell r="K99"/>
-          <cell r="L99"/>
-          <cell r="M99"/>
-          <cell r="N99"/>
-          <cell r="O99"/>
-          <cell r="P99"/>
-          <cell r="Q99"/>
-          <cell r="R99"/>
-          <cell r="S99"/>
-          <cell r="T99"/>
-          <cell r="U99"/>
-          <cell r="V99"/>
-          <cell r="W99"/>
-          <cell r="X99"/>
-        </row>
-        <row r="100">
-          <cell r="D100"/>
-          <cell r="E100"/>
-          <cell r="F100"/>
-          <cell r="G100"/>
-          <cell r="H100"/>
-          <cell r="I100"/>
-          <cell r="J100"/>
-          <cell r="K100"/>
-          <cell r="L100"/>
-          <cell r="M100"/>
-          <cell r="N100"/>
-          <cell r="O100"/>
-          <cell r="P100"/>
-          <cell r="Q100"/>
-          <cell r="R100"/>
-          <cell r="S100"/>
-          <cell r="T100"/>
-          <cell r="U100"/>
-          <cell r="V100"/>
-          <cell r="W100"/>
-          <cell r="X100"/>
-        </row>
-        <row r="101">
-          <cell r="D101"/>
-          <cell r="E101"/>
-          <cell r="F101"/>
-          <cell r="G101"/>
-          <cell r="H101"/>
-          <cell r="I101"/>
-          <cell r="J101"/>
-          <cell r="K101"/>
-          <cell r="L101"/>
-          <cell r="M101"/>
-          <cell r="N101"/>
-          <cell r="O101"/>
-          <cell r="P101"/>
-          <cell r="Q101"/>
-          <cell r="R101"/>
-          <cell r="S101"/>
-          <cell r="T101"/>
-          <cell r="U101"/>
-          <cell r="V101"/>
-          <cell r="W101"/>
-          <cell r="X101"/>
-        </row>
-        <row r="102">
-          <cell r="D102"/>
-          <cell r="E102"/>
-          <cell r="F102"/>
-          <cell r="G102"/>
-          <cell r="H102"/>
-          <cell r="I102"/>
-          <cell r="J102"/>
-          <cell r="K102"/>
-          <cell r="L102"/>
-          <cell r="M102"/>
-          <cell r="N102"/>
-          <cell r="O102"/>
-          <cell r="P102"/>
-          <cell r="Q102"/>
-          <cell r="R102"/>
-          <cell r="S102"/>
-          <cell r="T102"/>
-          <cell r="U102"/>
-          <cell r="V102"/>
-          <cell r="W102"/>
-          <cell r="X102"/>
-        </row>
-        <row r="103">
-          <cell r="D103"/>
-          <cell r="E103"/>
-          <cell r="F103"/>
-          <cell r="G103"/>
-          <cell r="H103"/>
-          <cell r="I103"/>
-          <cell r="J103"/>
-          <cell r="K103"/>
-          <cell r="L103"/>
-          <cell r="M103"/>
-          <cell r="N103"/>
-          <cell r="O103"/>
-          <cell r="P103"/>
-          <cell r="Q103"/>
-          <cell r="R103"/>
-          <cell r="S103"/>
-          <cell r="T103"/>
-          <cell r="U103"/>
-          <cell r="V103"/>
-          <cell r="W103"/>
-          <cell r="X103"/>
-        </row>
-        <row r="104">
-          <cell r="D104"/>
-          <cell r="E104"/>
-          <cell r="F104"/>
-          <cell r="G104"/>
-          <cell r="H104"/>
-          <cell r="I104"/>
-          <cell r="J104"/>
-          <cell r="K104"/>
-          <cell r="L104"/>
-          <cell r="M104"/>
-          <cell r="N104"/>
-          <cell r="O104"/>
-          <cell r="P104"/>
-          <cell r="Q104"/>
-          <cell r="R104"/>
-          <cell r="S104"/>
-          <cell r="T104"/>
-          <cell r="U104"/>
-          <cell r="V104"/>
-          <cell r="W104"/>
-          <cell r="X104"/>
-        </row>
-        <row r="105">
-          <cell r="D105"/>
-          <cell r="E105"/>
-          <cell r="F105"/>
-          <cell r="G105"/>
-          <cell r="H105"/>
-          <cell r="I105"/>
-          <cell r="J105"/>
-          <cell r="K105"/>
-          <cell r="L105"/>
-          <cell r="M105"/>
-          <cell r="N105"/>
-          <cell r="O105"/>
-          <cell r="P105"/>
-          <cell r="Q105"/>
-          <cell r="R105"/>
-          <cell r="S105"/>
-          <cell r="T105"/>
-          <cell r="U105"/>
-          <cell r="V105"/>
-          <cell r="W105"/>
-          <cell r="X105"/>
-        </row>
-        <row r="106">
-          <cell r="D106"/>
-          <cell r="E106"/>
-          <cell r="F106"/>
-          <cell r="G106"/>
-          <cell r="H106"/>
-          <cell r="I106"/>
-          <cell r="J106"/>
-          <cell r="K106"/>
-          <cell r="L106"/>
-          <cell r="M106"/>
-          <cell r="N106"/>
-          <cell r="O106"/>
-          <cell r="P106"/>
-          <cell r="Q106"/>
-          <cell r="R106"/>
-          <cell r="S106"/>
-          <cell r="T106"/>
-          <cell r="U106"/>
-          <cell r="V106"/>
-          <cell r="W106"/>
-          <cell r="X106"/>
-        </row>
-        <row r="107">
-          <cell r="D107"/>
-          <cell r="E107"/>
-          <cell r="F107"/>
-          <cell r="G107"/>
-          <cell r="H107"/>
-          <cell r="I107"/>
-          <cell r="J107"/>
-          <cell r="K107"/>
-          <cell r="L107"/>
-          <cell r="M107"/>
-          <cell r="N107"/>
-          <cell r="O107"/>
-          <cell r="P107"/>
-          <cell r="Q107"/>
-          <cell r="R107"/>
-          <cell r="S107"/>
-          <cell r="T107"/>
-          <cell r="U107"/>
-          <cell r="V107"/>
-          <cell r="W107"/>
-          <cell r="X107"/>
-        </row>
-        <row r="108">
-          <cell r="D108"/>
-          <cell r="E108"/>
-          <cell r="F108"/>
-          <cell r="G108"/>
-          <cell r="H108"/>
-          <cell r="I108"/>
-          <cell r="J108"/>
-          <cell r="K108"/>
-          <cell r="L108"/>
-          <cell r="M108"/>
-          <cell r="N108"/>
-          <cell r="O108"/>
-          <cell r="P108"/>
-          <cell r="Q108"/>
-          <cell r="R108"/>
-          <cell r="S108"/>
-          <cell r="T108"/>
-          <cell r="U108"/>
-          <cell r="V108"/>
-          <cell r="W108"/>
-          <cell r="X108"/>
-        </row>
-        <row r="109">
-          <cell r="D109"/>
-          <cell r="E109"/>
-          <cell r="F109"/>
-          <cell r="G109"/>
-          <cell r="H109"/>
-          <cell r="I109"/>
-          <cell r="J109"/>
-          <cell r="K109"/>
-          <cell r="L109"/>
-          <cell r="M109"/>
-          <cell r="N109"/>
-          <cell r="O109"/>
-          <cell r="P109"/>
-          <cell r="Q109"/>
-          <cell r="R109"/>
-          <cell r="S109"/>
-          <cell r="T109"/>
-          <cell r="U109"/>
-          <cell r="V109"/>
-          <cell r="W109"/>
-          <cell r="X109"/>
-        </row>
-        <row r="110">
-          <cell r="D110"/>
-          <cell r="E110"/>
-          <cell r="F110"/>
-          <cell r="G110"/>
-          <cell r="H110"/>
-          <cell r="I110"/>
-          <cell r="J110"/>
-          <cell r="K110"/>
-          <cell r="L110"/>
-          <cell r="M110"/>
-          <cell r="N110"/>
-          <cell r="O110"/>
-          <cell r="P110"/>
-          <cell r="Q110"/>
-          <cell r="R110"/>
-          <cell r="S110"/>
-          <cell r="T110"/>
-          <cell r="U110"/>
-          <cell r="V110"/>
-          <cell r="W110"/>
-          <cell r="X110"/>
-        </row>
-        <row r="111">
-          <cell r="D111"/>
-          <cell r="E111"/>
-          <cell r="F111"/>
-          <cell r="G111"/>
-          <cell r="H111"/>
-          <cell r="I111"/>
-          <cell r="J111"/>
-          <cell r="K111"/>
-          <cell r="L111"/>
-          <cell r="M111"/>
-          <cell r="N111"/>
-          <cell r="O111"/>
-          <cell r="P111"/>
-          <cell r="Q111"/>
-          <cell r="R111"/>
-          <cell r="S111"/>
-          <cell r="T111"/>
-          <cell r="U111"/>
-          <cell r="V111"/>
-          <cell r="W111"/>
-          <cell r="X111"/>
-        </row>
-        <row r="112">
-          <cell r="D112"/>
-          <cell r="E112"/>
-          <cell r="F112"/>
-          <cell r="G112"/>
-          <cell r="H112"/>
-          <cell r="I112"/>
-          <cell r="J112"/>
-          <cell r="K112"/>
-          <cell r="L112"/>
-          <cell r="M112"/>
-          <cell r="N112"/>
-          <cell r="O112"/>
-          <cell r="P112"/>
-          <cell r="Q112"/>
-          <cell r="R112"/>
-          <cell r="S112"/>
-          <cell r="T112"/>
-          <cell r="U112"/>
-          <cell r="V112"/>
-          <cell r="W112"/>
-          <cell r="X112"/>
-        </row>
-        <row r="113">
-          <cell r="D113"/>
-          <cell r="E113"/>
-          <cell r="F113"/>
-          <cell r="G113"/>
-          <cell r="H113"/>
-          <cell r="I113"/>
-          <cell r="J113"/>
-          <cell r="K113"/>
-          <cell r="L113"/>
-          <cell r="M113"/>
-          <cell r="N113"/>
-          <cell r="O113"/>
-          <cell r="P113"/>
-          <cell r="Q113"/>
-          <cell r="R113"/>
-          <cell r="S113"/>
-          <cell r="T113"/>
-          <cell r="U113"/>
-          <cell r="V113"/>
-          <cell r="W113"/>
-          <cell r="X113"/>
-        </row>
-        <row r="114">
-          <cell r="D114"/>
-          <cell r="E114"/>
-          <cell r="F114"/>
-          <cell r="G114"/>
-          <cell r="H114"/>
-          <cell r="I114"/>
-          <cell r="J114"/>
-          <cell r="K114"/>
-          <cell r="L114"/>
-          <cell r="M114"/>
-          <cell r="N114"/>
-          <cell r="O114"/>
-          <cell r="P114"/>
-          <cell r="Q114"/>
-          <cell r="R114"/>
-          <cell r="S114"/>
-          <cell r="T114"/>
-          <cell r="U114"/>
-          <cell r="V114"/>
-          <cell r="W114"/>
-          <cell r="X114"/>
-        </row>
-        <row r="115">
-          <cell r="D115"/>
-          <cell r="E115"/>
-          <cell r="F115"/>
-          <cell r="G115"/>
-          <cell r="H115"/>
-          <cell r="I115"/>
-          <cell r="J115"/>
-          <cell r="K115"/>
-          <cell r="L115"/>
-          <cell r="M115"/>
-          <cell r="N115"/>
-          <cell r="O115"/>
-          <cell r="P115"/>
-          <cell r="Q115"/>
-          <cell r="R115"/>
-          <cell r="S115"/>
-          <cell r="T115"/>
-          <cell r="U115"/>
-          <cell r="V115"/>
-          <cell r="W115"/>
-          <cell r="X115"/>
-        </row>
-        <row r="116">
-          <cell r="D116"/>
-          <cell r="E116"/>
-          <cell r="F116"/>
-          <cell r="G116"/>
-          <cell r="H116"/>
-          <cell r="I116"/>
-          <cell r="J116"/>
-          <cell r="K116"/>
-          <cell r="L116"/>
-          <cell r="M116"/>
-          <cell r="N116"/>
-          <cell r="O116"/>
-          <cell r="P116"/>
-          <cell r="Q116"/>
-          <cell r="R116"/>
-          <cell r="S116"/>
-          <cell r="T116"/>
-          <cell r="U116"/>
-          <cell r="V116"/>
-          <cell r="W116"/>
-          <cell r="X116"/>
-        </row>
-        <row r="117">
-          <cell r="D117"/>
-          <cell r="E117"/>
-          <cell r="F117"/>
-          <cell r="G117"/>
-          <cell r="H117"/>
-          <cell r="I117"/>
-          <cell r="J117"/>
-          <cell r="K117"/>
-          <cell r="L117"/>
-          <cell r="M117"/>
-          <cell r="N117"/>
-          <cell r="O117"/>
-          <cell r="P117"/>
-          <cell r="Q117"/>
-          <cell r="R117"/>
-          <cell r="S117"/>
-          <cell r="T117"/>
-          <cell r="U117"/>
-          <cell r="V117"/>
-          <cell r="W117"/>
-          <cell r="X117"/>
-        </row>
-        <row r="118">
-          <cell r="D118"/>
-          <cell r="E118"/>
-          <cell r="F118"/>
-          <cell r="G118"/>
-          <cell r="H118"/>
-          <cell r="I118"/>
-          <cell r="J118"/>
-          <cell r="K118"/>
-          <cell r="L118"/>
-          <cell r="M118"/>
-          <cell r="N118"/>
-          <cell r="O118"/>
-          <cell r="P118"/>
-          <cell r="Q118"/>
-          <cell r="R118"/>
-          <cell r="S118"/>
-          <cell r="T118"/>
-          <cell r="U118"/>
-          <cell r="V118"/>
-          <cell r="W118"/>
-          <cell r="X118"/>
-        </row>
-        <row r="119">
-          <cell r="D119"/>
-          <cell r="E119"/>
-          <cell r="F119"/>
-          <cell r="G119"/>
-          <cell r="H119"/>
-          <cell r="I119"/>
-          <cell r="J119"/>
-          <cell r="K119"/>
-          <cell r="L119"/>
-          <cell r="M119"/>
-          <cell r="N119"/>
-          <cell r="O119"/>
-          <cell r="P119"/>
-          <cell r="Q119"/>
-          <cell r="R119"/>
-          <cell r="S119"/>
-          <cell r="T119"/>
-          <cell r="U119"/>
-          <cell r="V119"/>
-          <cell r="W119"/>
-          <cell r="X119"/>
-        </row>
-        <row r="120">
-          <cell r="D120"/>
-          <cell r="E120"/>
-          <cell r="F120"/>
-          <cell r="G120"/>
-          <cell r="H120"/>
-          <cell r="I120"/>
-          <cell r="J120"/>
-          <cell r="K120"/>
-          <cell r="L120"/>
-          <cell r="M120"/>
-          <cell r="N120"/>
-          <cell r="O120"/>
-          <cell r="P120"/>
-          <cell r="Q120"/>
-          <cell r="R120"/>
-          <cell r="S120"/>
-          <cell r="T120"/>
-          <cell r="U120"/>
-          <cell r="V120"/>
-          <cell r="W120"/>
-          <cell r="X120"/>
-        </row>
-        <row r="121">
-          <cell r="D121"/>
-          <cell r="E121"/>
-          <cell r="F121"/>
-          <cell r="G121"/>
-          <cell r="H121"/>
-          <cell r="I121"/>
-          <cell r="J121"/>
-          <cell r="K121"/>
-          <cell r="L121"/>
-          <cell r="M121"/>
-          <cell r="N121"/>
-          <cell r="O121"/>
-          <cell r="P121"/>
-          <cell r="Q121"/>
-          <cell r="R121"/>
-          <cell r="S121"/>
-          <cell r="T121"/>
-          <cell r="U121"/>
-          <cell r="V121"/>
-          <cell r="W121"/>
-          <cell r="X121"/>
-        </row>
-        <row r="122">
-          <cell r="D122"/>
-          <cell r="E122"/>
-          <cell r="F122"/>
-          <cell r="G122"/>
-          <cell r="H122"/>
-          <cell r="I122"/>
-          <cell r="J122"/>
-          <cell r="K122"/>
-          <cell r="L122"/>
-          <cell r="M122"/>
-          <cell r="N122"/>
-          <cell r="O122"/>
-          <cell r="P122"/>
-          <cell r="Q122"/>
-          <cell r="R122"/>
-          <cell r="S122"/>
-          <cell r="T122"/>
-          <cell r="U122"/>
-          <cell r="V122"/>
-          <cell r="W122"/>
-          <cell r="X122"/>
-        </row>
-        <row r="123">
-          <cell r="D123"/>
-          <cell r="E123"/>
-          <cell r="F123"/>
-          <cell r="G123"/>
-          <cell r="H123"/>
-          <cell r="I123"/>
-          <cell r="J123"/>
-          <cell r="K123"/>
-          <cell r="L123"/>
-          <cell r="M123"/>
-          <cell r="N123"/>
-          <cell r="O123"/>
-          <cell r="P123"/>
-          <cell r="Q123"/>
-          <cell r="R123"/>
-          <cell r="S123"/>
-          <cell r="T123"/>
-          <cell r="U123"/>
-          <cell r="V123"/>
-          <cell r="W123"/>
-          <cell r="X123"/>
-        </row>
-        <row r="124">
-          <cell r="D124"/>
-          <cell r="E124"/>
-          <cell r="F124"/>
-          <cell r="G124"/>
-          <cell r="H124"/>
-          <cell r="I124"/>
-          <cell r="J124"/>
-          <cell r="K124"/>
-          <cell r="L124"/>
-          <cell r="M124"/>
-          <cell r="N124"/>
-          <cell r="O124"/>
-          <cell r="P124"/>
-          <cell r="Q124"/>
-          <cell r="R124"/>
-          <cell r="S124"/>
-          <cell r="T124"/>
-          <cell r="U124"/>
-          <cell r="V124"/>
-          <cell r="W124"/>
-          <cell r="X124"/>
-        </row>
-        <row r="125">
-          <cell r="D125"/>
-          <cell r="E125"/>
-          <cell r="F125"/>
-          <cell r="G125"/>
-          <cell r="H125"/>
-          <cell r="I125"/>
-          <cell r="J125"/>
-          <cell r="K125"/>
-          <cell r="L125"/>
-          <cell r="M125"/>
-          <cell r="N125"/>
-          <cell r="O125"/>
-          <cell r="P125"/>
-          <cell r="Q125"/>
-          <cell r="R125"/>
-          <cell r="S125"/>
-          <cell r="T125"/>
-          <cell r="U125"/>
-          <cell r="V125"/>
-          <cell r="W125"/>
-          <cell r="X125"/>
-        </row>
-        <row r="126">
-          <cell r="D126"/>
-          <cell r="E126"/>
-          <cell r="F126"/>
-          <cell r="G126"/>
-          <cell r="H126"/>
-          <cell r="I126"/>
-          <cell r="J126"/>
-          <cell r="K126"/>
-          <cell r="L126"/>
-          <cell r="M126"/>
-          <cell r="N126"/>
-          <cell r="O126"/>
-          <cell r="P126"/>
-          <cell r="Q126"/>
-          <cell r="R126"/>
-          <cell r="S126"/>
-          <cell r="T126"/>
-          <cell r="U126"/>
-          <cell r="V126"/>
-          <cell r="W126"/>
-          <cell r="X126"/>
-        </row>
-        <row r="127">
-          <cell r="D127"/>
-          <cell r="E127"/>
-          <cell r="F127"/>
-          <cell r="G127"/>
-          <cell r="H127"/>
-          <cell r="I127"/>
-          <cell r="J127"/>
-          <cell r="K127"/>
-          <cell r="L127"/>
-          <cell r="M127"/>
-          <cell r="N127"/>
-          <cell r="O127"/>
-          <cell r="P127"/>
-          <cell r="Q127"/>
-          <cell r="R127"/>
-          <cell r="S127"/>
-          <cell r="T127"/>
-          <cell r="U127"/>
-          <cell r="V127"/>
-          <cell r="W127"/>
-          <cell r="X127"/>
-        </row>
-        <row r="128">
-          <cell r="D128"/>
-          <cell r="E128"/>
-          <cell r="F128"/>
-          <cell r="G128"/>
-          <cell r="H128"/>
-          <cell r="I128"/>
-          <cell r="J128"/>
-          <cell r="K128"/>
-          <cell r="L128"/>
-          <cell r="M128"/>
-          <cell r="N128"/>
-          <cell r="O128"/>
-          <cell r="P128"/>
-          <cell r="Q128"/>
-          <cell r="R128"/>
-          <cell r="S128"/>
-          <cell r="T128"/>
-          <cell r="U128"/>
-          <cell r="V128"/>
-          <cell r="W128"/>
-          <cell r="X128"/>
-        </row>
-        <row r="129">
-          <cell r="D129"/>
-          <cell r="E129"/>
-          <cell r="F129"/>
-          <cell r="G129"/>
-          <cell r="H129"/>
-          <cell r="I129"/>
-          <cell r="J129"/>
-          <cell r="K129"/>
-          <cell r="L129"/>
-          <cell r="M129"/>
-          <cell r="N129"/>
-          <cell r="O129"/>
-          <cell r="P129"/>
-          <cell r="Q129"/>
-          <cell r="R129"/>
-          <cell r="S129"/>
-          <cell r="T129"/>
-          <cell r="U129"/>
-          <cell r="V129"/>
-          <cell r="W129"/>
-          <cell r="X129"/>
-        </row>
-        <row r="130">
-          <cell r="D130"/>
-          <cell r="E130"/>
-          <cell r="F130"/>
-          <cell r="G130"/>
-          <cell r="H130"/>
-          <cell r="I130"/>
-          <cell r="J130"/>
-          <cell r="K130"/>
-          <cell r="L130"/>
-          <cell r="M130"/>
-          <cell r="N130"/>
-          <cell r="O130"/>
-          <cell r="P130"/>
-          <cell r="Q130"/>
-          <cell r="R130"/>
-          <cell r="S130"/>
-          <cell r="T130"/>
-          <cell r="U130"/>
-          <cell r="V130"/>
-          <cell r="W130"/>
-          <cell r="X130"/>
-        </row>
-        <row r="131">
-          <cell r="D131"/>
-          <cell r="E131"/>
-          <cell r="F131"/>
-          <cell r="G131"/>
-          <cell r="H131"/>
-          <cell r="I131"/>
-          <cell r="J131"/>
-          <cell r="K131"/>
-          <cell r="L131"/>
-          <cell r="M131"/>
-          <cell r="N131"/>
-          <cell r="O131"/>
-          <cell r="P131"/>
-          <cell r="Q131"/>
-          <cell r="R131"/>
-          <cell r="S131"/>
-          <cell r="T131"/>
-          <cell r="U131"/>
-          <cell r="V131"/>
-          <cell r="W131"/>
-          <cell r="X131"/>
-        </row>
-        <row r="132">
-          <cell r="D132"/>
-          <cell r="E132"/>
-          <cell r="F132"/>
-          <cell r="G132"/>
-          <cell r="H132"/>
-          <cell r="I132"/>
-          <cell r="J132"/>
-          <cell r="K132"/>
-          <cell r="L132"/>
-          <cell r="M132"/>
-          <cell r="N132"/>
-          <cell r="O132"/>
-          <cell r="P132"/>
-          <cell r="Q132"/>
-          <cell r="R132"/>
-          <cell r="S132"/>
-          <cell r="T132"/>
-          <cell r="U132"/>
-          <cell r="V132"/>
-          <cell r="W132"/>
-          <cell r="X132"/>
-        </row>
-        <row r="133">
-          <cell r="D133"/>
-          <cell r="E133"/>
-          <cell r="F133"/>
-          <cell r="G133"/>
-          <cell r="H133"/>
-          <cell r="I133"/>
-          <cell r="J133"/>
-          <cell r="K133"/>
-          <cell r="L133"/>
-          <cell r="M133"/>
-          <cell r="N133"/>
-          <cell r="O133"/>
-          <cell r="P133"/>
-          <cell r="Q133"/>
-          <cell r="R133"/>
-          <cell r="S133"/>
-          <cell r="T133"/>
-          <cell r="U133"/>
-          <cell r="V133"/>
-          <cell r="W133"/>
-          <cell r="X133"/>
-        </row>
-        <row r="134">
-          <cell r="D134"/>
-          <cell r="E134"/>
-          <cell r="F134"/>
-          <cell r="G134"/>
-          <cell r="H134"/>
-          <cell r="I134"/>
-          <cell r="J134"/>
-          <cell r="K134"/>
-          <cell r="L134"/>
-          <cell r="M134"/>
-          <cell r="N134"/>
-          <cell r="O134"/>
-          <cell r="P134"/>
-          <cell r="Q134"/>
-          <cell r="R134"/>
-          <cell r="S134"/>
-          <cell r="T134"/>
-          <cell r="U134"/>
-          <cell r="V134"/>
-          <cell r="W134"/>
-          <cell r="X134"/>
-        </row>
-        <row r="135">
-          <cell r="D135"/>
-          <cell r="E135"/>
-          <cell r="F135"/>
-          <cell r="G135"/>
-          <cell r="H135"/>
-          <cell r="I135"/>
-          <cell r="J135"/>
-          <cell r="K135"/>
-          <cell r="L135"/>
-          <cell r="M135"/>
-          <cell r="N135"/>
-          <cell r="O135"/>
-          <cell r="P135"/>
-          <cell r="Q135"/>
-          <cell r="R135"/>
-          <cell r="S135"/>
-          <cell r="T135"/>
-          <cell r="U135"/>
-          <cell r="V135"/>
-          <cell r="W135"/>
-          <cell r="X135"/>
-        </row>
-        <row r="136">
-          <cell r="D136"/>
-          <cell r="E136"/>
-          <cell r="F136"/>
-          <cell r="G136"/>
-          <cell r="H136"/>
-          <cell r="I136"/>
-          <cell r="J136"/>
-          <cell r="K136"/>
-          <cell r="L136"/>
-          <cell r="M136"/>
-          <cell r="N136"/>
-          <cell r="O136"/>
-          <cell r="P136"/>
-          <cell r="Q136"/>
-          <cell r="R136"/>
-          <cell r="S136"/>
-          <cell r="T136"/>
-          <cell r="U136"/>
-          <cell r="V136"/>
-          <cell r="W136"/>
-          <cell r="X136"/>
-        </row>
-        <row r="137">
-          <cell r="D137"/>
-          <cell r="E137"/>
-          <cell r="F137"/>
-          <cell r="G137"/>
-          <cell r="H137"/>
-          <cell r="I137"/>
-          <cell r="J137"/>
-          <cell r="K137"/>
-          <cell r="L137"/>
-          <cell r="M137"/>
-          <cell r="N137"/>
-          <cell r="O137"/>
-          <cell r="P137"/>
-          <cell r="Q137"/>
-          <cell r="R137"/>
-          <cell r="S137"/>
-          <cell r="T137"/>
-          <cell r="U137"/>
-          <cell r="V137"/>
-          <cell r="W137"/>
-          <cell r="X137"/>
-        </row>
-        <row r="138">
-          <cell r="D138"/>
-          <cell r="E138"/>
-          <cell r="F138"/>
-          <cell r="G138"/>
-          <cell r="H138"/>
-          <cell r="I138"/>
-          <cell r="J138"/>
-          <cell r="K138"/>
-          <cell r="L138"/>
-          <cell r="M138"/>
-          <cell r="N138"/>
-          <cell r="O138"/>
-          <cell r="P138"/>
-          <cell r="Q138"/>
-          <cell r="R138"/>
-          <cell r="S138"/>
-          <cell r="T138"/>
-          <cell r="U138"/>
-          <cell r="V138"/>
-          <cell r="W138"/>
-          <cell r="X138"/>
-        </row>
-        <row r="139">
-          <cell r="D139"/>
-          <cell r="E139"/>
-          <cell r="F139"/>
-          <cell r="G139"/>
-          <cell r="H139"/>
-          <cell r="I139"/>
-          <cell r="J139"/>
-          <cell r="K139"/>
-          <cell r="L139"/>
-          <cell r="M139"/>
-          <cell r="N139"/>
-          <cell r="O139"/>
-          <cell r="P139"/>
-          <cell r="Q139"/>
-          <cell r="R139"/>
-          <cell r="S139"/>
-          <cell r="T139"/>
-          <cell r="U139"/>
-          <cell r="V139"/>
-          <cell r="W139"/>
-          <cell r="X139"/>
-        </row>
-        <row r="140">
-          <cell r="D140"/>
-          <cell r="E140"/>
-          <cell r="F140"/>
-          <cell r="G140"/>
-          <cell r="H140"/>
-          <cell r="I140"/>
-          <cell r="J140"/>
-          <cell r="K140"/>
-          <cell r="L140"/>
-          <cell r="M140"/>
-          <cell r="N140"/>
-          <cell r="O140"/>
-          <cell r="P140"/>
-          <cell r="Q140"/>
-          <cell r="R140"/>
-          <cell r="S140"/>
-          <cell r="T140"/>
-          <cell r="U140"/>
-          <cell r="V140"/>
-          <cell r="W140"/>
-          <cell r="X140"/>
-        </row>
-        <row r="141">
-          <cell r="D141"/>
-          <cell r="E141"/>
-          <cell r="F141"/>
-          <cell r="G141"/>
-          <cell r="H141"/>
-          <cell r="I141"/>
-          <cell r="J141"/>
-          <cell r="K141"/>
-          <cell r="L141"/>
-          <cell r="M141"/>
-          <cell r="N141"/>
-          <cell r="O141"/>
-          <cell r="P141"/>
-          <cell r="Q141"/>
-          <cell r="R141"/>
-          <cell r="S141"/>
-          <cell r="T141"/>
-          <cell r="U141"/>
-          <cell r="V141"/>
-          <cell r="W141"/>
-          <cell r="X141"/>
-        </row>
-        <row r="142">
-          <cell r="D142"/>
-          <cell r="E142"/>
-          <cell r="F142"/>
-          <cell r="G142"/>
-          <cell r="H142"/>
-          <cell r="I142"/>
-          <cell r="J142"/>
-          <cell r="K142"/>
-          <cell r="L142"/>
-          <cell r="M142"/>
-          <cell r="N142"/>
-          <cell r="O142"/>
-          <cell r="P142"/>
-          <cell r="Q142"/>
-          <cell r="R142"/>
-          <cell r="S142"/>
-          <cell r="T142"/>
-          <cell r="U142"/>
-          <cell r="V142"/>
-          <cell r="W142"/>
-          <cell r="X142"/>
-        </row>
-        <row r="143">
-          <cell r="D143"/>
-          <cell r="E143"/>
-          <cell r="F143"/>
-          <cell r="G143"/>
-          <cell r="H143"/>
-          <cell r="I143"/>
-          <cell r="J143"/>
-          <cell r="K143"/>
-          <cell r="L143"/>
-          <cell r="M143"/>
-          <cell r="N143"/>
-          <cell r="O143"/>
-          <cell r="P143"/>
-          <cell r="Q143"/>
-          <cell r="R143"/>
-          <cell r="S143"/>
-          <cell r="T143"/>
-          <cell r="U143"/>
-          <cell r="V143"/>
-          <cell r="W143"/>
-          <cell r="X143"/>
-        </row>
-        <row r="144">
-          <cell r="D144"/>
-          <cell r="E144"/>
-          <cell r="F144"/>
-          <cell r="G144"/>
-          <cell r="H144"/>
-          <cell r="I144"/>
-          <cell r="J144"/>
-          <cell r="K144"/>
-          <cell r="L144"/>
-          <cell r="M144"/>
-          <cell r="N144"/>
-          <cell r="O144"/>
-          <cell r="P144"/>
-          <cell r="Q144"/>
-          <cell r="R144"/>
-          <cell r="S144"/>
-          <cell r="T144"/>
-          <cell r="U144"/>
-          <cell r="V144"/>
-          <cell r="W144"/>
-          <cell r="X144"/>
-        </row>
-        <row r="145">
-          <cell r="D145"/>
-          <cell r="E145"/>
-          <cell r="F145"/>
-          <cell r="G145"/>
-          <cell r="H145"/>
-          <cell r="I145"/>
-          <cell r="J145"/>
-          <cell r="K145"/>
-          <cell r="L145"/>
-          <cell r="M145"/>
-          <cell r="N145"/>
-          <cell r="O145"/>
-          <cell r="P145"/>
-          <cell r="Q145"/>
-          <cell r="R145"/>
-          <cell r="S145"/>
-          <cell r="T145"/>
-          <cell r="U145"/>
-          <cell r="V145"/>
-          <cell r="W145"/>
-          <cell r="X145"/>
-        </row>
-        <row r="146">
-          <cell r="D146"/>
-          <cell r="E146"/>
-          <cell r="F146"/>
-          <cell r="G146"/>
-          <cell r="H146"/>
-          <cell r="I146"/>
-          <cell r="J146"/>
-          <cell r="K146"/>
-          <cell r="L146"/>
-          <cell r="M146"/>
-          <cell r="N146"/>
-          <cell r="O146"/>
-          <cell r="P146"/>
-          <cell r="Q146"/>
-          <cell r="R146"/>
-          <cell r="S146"/>
-          <cell r="T146"/>
-          <cell r="U146"/>
-          <cell r="V146"/>
-          <cell r="W146"/>
-          <cell r="X146"/>
-        </row>
-        <row r="147">
-          <cell r="D147"/>
-          <cell r="E147"/>
-          <cell r="F147"/>
-          <cell r="G147"/>
-          <cell r="H147"/>
-          <cell r="I147"/>
-          <cell r="J147"/>
-          <cell r="K147"/>
-          <cell r="L147"/>
-          <cell r="M147"/>
-          <cell r="N147"/>
-          <cell r="O147"/>
-          <cell r="P147"/>
-          <cell r="Q147"/>
-          <cell r="R147"/>
-          <cell r="S147"/>
-          <cell r="T147"/>
-          <cell r="U147"/>
-          <cell r="V147"/>
-          <cell r="W147"/>
-          <cell r="X147"/>
-        </row>
-        <row r="148">
-          <cell r="D148"/>
-          <cell r="E148"/>
-          <cell r="F148"/>
-          <cell r="G148"/>
-          <cell r="H148"/>
-          <cell r="I148"/>
-          <cell r="J148"/>
-          <cell r="K148"/>
-          <cell r="L148"/>
-          <cell r="M148"/>
-          <cell r="N148"/>
-          <cell r="O148"/>
-          <cell r="P148"/>
-          <cell r="Q148"/>
-          <cell r="R148"/>
-          <cell r="S148"/>
-          <cell r="T148"/>
-          <cell r="U148"/>
-          <cell r="V148"/>
-          <cell r="W148"/>
-          <cell r="X148"/>
-        </row>
-        <row r="149">
-          <cell r="D149"/>
-          <cell r="E149"/>
-          <cell r="F149"/>
-          <cell r="G149"/>
-          <cell r="H149"/>
-          <cell r="I149"/>
-          <cell r="J149"/>
-          <cell r="K149"/>
-          <cell r="L149"/>
-          <cell r="M149"/>
-          <cell r="N149"/>
-          <cell r="O149"/>
-          <cell r="P149"/>
-          <cell r="Q149"/>
-          <cell r="R149"/>
-          <cell r="S149"/>
-          <cell r="T149"/>
-          <cell r="U149"/>
-          <cell r="V149"/>
-          <cell r="W149"/>
-          <cell r="X149"/>
-        </row>
-        <row r="150">
-          <cell r="D150"/>
-          <cell r="E150"/>
-          <cell r="F150"/>
-          <cell r="G150"/>
-          <cell r="H150"/>
-          <cell r="I150"/>
-          <cell r="J150"/>
-          <cell r="K150"/>
-          <cell r="L150"/>
-          <cell r="M150"/>
-          <cell r="N150"/>
-          <cell r="O150"/>
-          <cell r="P150"/>
-          <cell r="Q150"/>
-          <cell r="R150"/>
-          <cell r="S150"/>
-          <cell r="T150"/>
-          <cell r="U150"/>
-          <cell r="V150"/>
-          <cell r="W150"/>
-          <cell r="X150"/>
-        </row>
-        <row r="151">
-          <cell r="D151"/>
-          <cell r="E151"/>
-          <cell r="F151"/>
-          <cell r="G151"/>
-          <cell r="H151"/>
-          <cell r="I151"/>
-          <cell r="J151"/>
-          <cell r="K151"/>
-          <cell r="L151"/>
-          <cell r="M151"/>
-          <cell r="N151"/>
-          <cell r="O151"/>
-          <cell r="P151"/>
-          <cell r="Q151"/>
-          <cell r="R151"/>
-          <cell r="S151"/>
-          <cell r="T151"/>
-          <cell r="U151"/>
-          <cell r="V151"/>
-          <cell r="W151"/>
-          <cell r="X151"/>
-        </row>
-        <row r="152">
-          <cell r="D152"/>
-          <cell r="E152"/>
-          <cell r="F152"/>
-          <cell r="G152"/>
-          <cell r="H152"/>
-          <cell r="I152"/>
-          <cell r="J152"/>
-          <cell r="K152"/>
-          <cell r="L152"/>
-          <cell r="M152"/>
-          <cell r="N152"/>
-          <cell r="O152"/>
-          <cell r="P152"/>
-          <cell r="Q152"/>
-          <cell r="R152"/>
-          <cell r="S152"/>
-          <cell r="T152"/>
-          <cell r="U152"/>
-          <cell r="V152"/>
-          <cell r="W152"/>
-          <cell r="X152"/>
-        </row>
-        <row r="153">
-          <cell r="D153"/>
-          <cell r="E153"/>
-          <cell r="F153"/>
-          <cell r="G153"/>
-          <cell r="H153"/>
-          <cell r="I153"/>
-          <cell r="J153"/>
-          <cell r="K153"/>
-          <cell r="L153"/>
-          <cell r="M153"/>
-          <cell r="N153"/>
-          <cell r="O153"/>
-          <cell r="P153"/>
-          <cell r="Q153"/>
-          <cell r="R153"/>
-          <cell r="S153"/>
-          <cell r="T153"/>
-          <cell r="U153"/>
-          <cell r="V153"/>
-          <cell r="W153"/>
-          <cell r="X153"/>
-        </row>
-        <row r="154">
-          <cell r="D154"/>
-          <cell r="E154"/>
-          <cell r="F154"/>
-          <cell r="G154"/>
-          <cell r="H154"/>
-          <cell r="I154"/>
-          <cell r="J154"/>
-          <cell r="K154"/>
-          <cell r="L154"/>
-          <cell r="M154"/>
-          <cell r="N154"/>
-          <cell r="O154"/>
-          <cell r="P154"/>
-          <cell r="Q154"/>
-          <cell r="R154"/>
-          <cell r="S154"/>
-          <cell r="T154"/>
-          <cell r="U154"/>
-          <cell r="V154"/>
-          <cell r="W154"/>
-          <cell r="X154"/>
-        </row>
-        <row r="155">
-          <cell r="D155"/>
-          <cell r="E155"/>
-          <cell r="F155"/>
-          <cell r="G155"/>
-          <cell r="H155"/>
-          <cell r="I155"/>
-          <cell r="J155"/>
-          <cell r="K155"/>
-          <cell r="L155"/>
-          <cell r="M155"/>
-          <cell r="N155"/>
-          <cell r="O155"/>
-          <cell r="P155"/>
-          <cell r="Q155"/>
-          <cell r="R155"/>
-          <cell r="S155"/>
-          <cell r="T155"/>
-          <cell r="U155"/>
-          <cell r="V155"/>
-          <cell r="W155"/>
-          <cell r="X155"/>
-        </row>
-        <row r="156">
-          <cell r="D156"/>
-          <cell r="E156"/>
-          <cell r="F156"/>
-          <cell r="G156"/>
-          <cell r="H156"/>
-          <cell r="I156"/>
-          <cell r="J156"/>
-          <cell r="K156"/>
-          <cell r="L156"/>
-          <cell r="M156"/>
-          <cell r="N156"/>
-          <cell r="O156"/>
-          <cell r="P156"/>
-          <cell r="Q156"/>
-          <cell r="R156"/>
-          <cell r="S156"/>
-          <cell r="T156"/>
-          <cell r="U156"/>
-          <cell r="V156"/>
-          <cell r="W156"/>
-          <cell r="X156"/>
-        </row>
-        <row r="157">
-          <cell r="D157"/>
-          <cell r="E157"/>
-          <cell r="F157"/>
-          <cell r="G157"/>
-          <cell r="H157"/>
-          <cell r="I157"/>
-          <cell r="J157"/>
-          <cell r="K157"/>
-          <cell r="L157"/>
-          <cell r="M157"/>
-          <cell r="N157"/>
-          <cell r="O157"/>
-          <cell r="P157"/>
-          <cell r="Q157"/>
-          <cell r="R157"/>
-          <cell r="S157"/>
-          <cell r="T157"/>
-          <cell r="U157"/>
-          <cell r="V157"/>
-          <cell r="W157"/>
-          <cell r="X157"/>
-        </row>
-        <row r="158">
-          <cell r="D158"/>
-          <cell r="E158"/>
-          <cell r="F158"/>
-          <cell r="G158"/>
-          <cell r="H158"/>
-          <cell r="I158"/>
-          <cell r="J158"/>
-          <cell r="K158"/>
-          <cell r="L158"/>
-          <cell r="M158"/>
-          <cell r="N158"/>
-          <cell r="O158"/>
-          <cell r="P158"/>
-          <cell r="Q158"/>
-          <cell r="R158"/>
-          <cell r="S158"/>
-          <cell r="T158"/>
-          <cell r="U158"/>
-          <cell r="V158"/>
-          <cell r="W158"/>
-          <cell r="X158"/>
-        </row>
-        <row r="159">
-          <cell r="D159"/>
-          <cell r="E159"/>
-          <cell r="F159"/>
-          <cell r="G159"/>
-          <cell r="H159"/>
-          <cell r="I159"/>
-          <cell r="J159"/>
-          <cell r="K159"/>
-          <cell r="L159"/>
-          <cell r="M159"/>
-          <cell r="N159"/>
-          <cell r="O159"/>
-          <cell r="P159"/>
-          <cell r="Q159"/>
-          <cell r="R159"/>
-          <cell r="S159"/>
-          <cell r="T159"/>
-          <cell r="U159"/>
-          <cell r="V159"/>
-          <cell r="W159"/>
-          <cell r="X159"/>
-        </row>
-        <row r="160">
-          <cell r="D160"/>
-          <cell r="E160"/>
-          <cell r="F160"/>
-          <cell r="G160"/>
-          <cell r="H160"/>
-          <cell r="I160"/>
-          <cell r="J160"/>
-          <cell r="K160"/>
-          <cell r="L160"/>
-          <cell r="M160"/>
-          <cell r="N160"/>
-          <cell r="O160"/>
-          <cell r="P160"/>
-          <cell r="Q160"/>
-          <cell r="R160"/>
-          <cell r="S160"/>
-          <cell r="T160"/>
-          <cell r="U160"/>
-          <cell r="V160"/>
-          <cell r="W160"/>
-          <cell r="X160"/>
-        </row>
-        <row r="161">
-          <cell r="D161"/>
-          <cell r="E161"/>
-          <cell r="F161"/>
-          <cell r="G161"/>
-          <cell r="H161"/>
-          <cell r="I161"/>
-          <cell r="J161"/>
-          <cell r="K161"/>
-          <cell r="L161"/>
-          <cell r="M161"/>
-          <cell r="N161"/>
-          <cell r="O161"/>
-          <cell r="P161"/>
-          <cell r="Q161"/>
-          <cell r="R161"/>
-          <cell r="S161"/>
-          <cell r="T161"/>
-          <cell r="U161"/>
-          <cell r="V161"/>
-          <cell r="W161"/>
-          <cell r="X161"/>
-        </row>
-        <row r="162">
-          <cell r="D162"/>
-          <cell r="E162"/>
-          <cell r="F162"/>
-          <cell r="G162"/>
-          <cell r="H162"/>
-          <cell r="I162"/>
-          <cell r="J162"/>
-          <cell r="K162"/>
-          <cell r="L162"/>
-          <cell r="M162"/>
-          <cell r="N162"/>
-          <cell r="O162"/>
-          <cell r="P162"/>
-          <cell r="Q162"/>
-          <cell r="R162"/>
-          <cell r="S162"/>
-          <cell r="T162"/>
-          <cell r="U162"/>
-          <cell r="V162"/>
-          <cell r="W162"/>
-          <cell r="X162"/>
-        </row>
-        <row r="163">
-          <cell r="D163"/>
-          <cell r="E163"/>
-          <cell r="F163"/>
-          <cell r="G163"/>
-          <cell r="H163"/>
-          <cell r="I163"/>
-          <cell r="J163"/>
-          <cell r="K163"/>
-          <cell r="L163"/>
-          <cell r="M163"/>
-          <cell r="N163"/>
-          <cell r="O163"/>
-          <cell r="P163"/>
-          <cell r="Q163"/>
-          <cell r="R163"/>
-          <cell r="S163"/>
-          <cell r="T163"/>
-          <cell r="U163"/>
-          <cell r="V163"/>
-          <cell r="W163"/>
-          <cell r="X163"/>
-        </row>
-        <row r="164">
-          <cell r="D164"/>
-          <cell r="E164"/>
-          <cell r="F164"/>
-          <cell r="G164"/>
-          <cell r="H164"/>
-          <cell r="I164"/>
-          <cell r="J164"/>
-          <cell r="K164"/>
-          <cell r="L164"/>
-          <cell r="M164"/>
-          <cell r="N164"/>
-          <cell r="O164"/>
-          <cell r="P164"/>
-          <cell r="Q164"/>
-          <cell r="R164"/>
-          <cell r="S164"/>
-          <cell r="T164"/>
-          <cell r="U164"/>
-          <cell r="V164"/>
-          <cell r="W164"/>
-          <cell r="X164"/>
-        </row>
-        <row r="165">
-          <cell r="D165"/>
-          <cell r="E165"/>
-          <cell r="F165"/>
-          <cell r="G165"/>
-          <cell r="H165"/>
-          <cell r="I165"/>
-          <cell r="J165"/>
-          <cell r="K165"/>
-          <cell r="L165"/>
-          <cell r="M165"/>
-          <cell r="N165"/>
-          <cell r="O165"/>
-          <cell r="P165"/>
-          <cell r="Q165"/>
-          <cell r="R165"/>
-          <cell r="S165"/>
-          <cell r="T165"/>
-          <cell r="U165"/>
-          <cell r="V165"/>
-          <cell r="W165"/>
-          <cell r="X165"/>
-        </row>
-        <row r="166">
-          <cell r="D166"/>
-          <cell r="E166"/>
-          <cell r="F166"/>
-          <cell r="G166"/>
-          <cell r="H166"/>
-          <cell r="I166"/>
-          <cell r="J166"/>
-          <cell r="K166"/>
-          <cell r="L166"/>
-          <cell r="M166"/>
-          <cell r="N166"/>
-          <cell r="O166"/>
-          <cell r="P166"/>
-          <cell r="Q166"/>
-          <cell r="R166"/>
-          <cell r="S166"/>
-          <cell r="T166"/>
-          <cell r="U166"/>
-          <cell r="V166"/>
-          <cell r="W166"/>
-          <cell r="X166"/>
-        </row>
-        <row r="167">
-          <cell r="D167"/>
-          <cell r="E167"/>
-          <cell r="F167"/>
-          <cell r="G167"/>
-          <cell r="H167"/>
-          <cell r="I167"/>
-          <cell r="J167"/>
-          <cell r="K167"/>
-          <cell r="L167"/>
-          <cell r="M167"/>
-          <cell r="N167"/>
-          <cell r="O167"/>
-          <cell r="P167"/>
-          <cell r="Q167"/>
-          <cell r="R167"/>
-          <cell r="S167"/>
-          <cell r="T167"/>
-          <cell r="U167"/>
-          <cell r="V167"/>
-          <cell r="W167"/>
-          <cell r="X167"/>
-        </row>
-        <row r="168">
-          <cell r="D168"/>
-          <cell r="E168"/>
-          <cell r="F168"/>
-          <cell r="G168"/>
-          <cell r="H168"/>
-          <cell r="I168"/>
-          <cell r="J168"/>
-          <cell r="K168"/>
-          <cell r="L168"/>
-          <cell r="M168"/>
-          <cell r="N168"/>
-          <cell r="O168"/>
-          <cell r="P168"/>
-          <cell r="Q168"/>
-          <cell r="R168"/>
-          <cell r="S168"/>
-          <cell r="T168"/>
-          <cell r="U168"/>
-          <cell r="V168"/>
-          <cell r="W168"/>
-          <cell r="X168"/>
-        </row>
-        <row r="169">
-          <cell r="D169"/>
-          <cell r="E169"/>
-          <cell r="F169"/>
-          <cell r="G169"/>
-          <cell r="H169"/>
-          <cell r="I169"/>
-          <cell r="J169"/>
-          <cell r="K169"/>
-          <cell r="L169"/>
-          <cell r="M169"/>
-          <cell r="N169"/>
-          <cell r="O169"/>
-          <cell r="P169"/>
-          <cell r="Q169"/>
-          <cell r="R169"/>
-          <cell r="S169"/>
-          <cell r="T169"/>
-          <cell r="U169"/>
-          <cell r="V169"/>
-          <cell r="W169"/>
-          <cell r="X169"/>
-        </row>
-        <row r="170">
-          <cell r="D170"/>
-          <cell r="E170"/>
-          <cell r="F170"/>
-          <cell r="G170"/>
-          <cell r="H170"/>
-          <cell r="I170"/>
-          <cell r="J170"/>
-          <cell r="K170"/>
-          <cell r="L170"/>
-          <cell r="M170"/>
-          <cell r="N170"/>
-          <cell r="O170"/>
-          <cell r="P170"/>
-          <cell r="Q170"/>
-          <cell r="R170"/>
-          <cell r="S170"/>
-          <cell r="T170"/>
-          <cell r="U170"/>
-          <cell r="V170"/>
-          <cell r="W170"/>
-          <cell r="X170"/>
-        </row>
-        <row r="171">
-          <cell r="D171"/>
-          <cell r="E171"/>
-          <cell r="F171"/>
-          <cell r="G171"/>
-          <cell r="H171"/>
-          <cell r="I171"/>
-          <cell r="J171"/>
-          <cell r="K171"/>
-          <cell r="L171"/>
-          <cell r="M171"/>
-          <cell r="N171"/>
-          <cell r="O171"/>
-          <cell r="P171"/>
-          <cell r="Q171"/>
-          <cell r="R171"/>
-          <cell r="S171"/>
-          <cell r="T171"/>
-          <cell r="U171"/>
-          <cell r="V171"/>
-          <cell r="W171"/>
-          <cell r="X171"/>
-        </row>
-        <row r="172">
-          <cell r="D172"/>
-          <cell r="E172"/>
-          <cell r="F172"/>
-          <cell r="G172"/>
-          <cell r="H172"/>
-          <cell r="I172"/>
-          <cell r="J172"/>
-          <cell r="K172"/>
-          <cell r="L172"/>
-          <cell r="M172"/>
-          <cell r="N172"/>
-          <cell r="O172"/>
-          <cell r="P172"/>
-          <cell r="Q172"/>
-          <cell r="R172"/>
-          <cell r="S172"/>
-          <cell r="T172"/>
-          <cell r="U172"/>
-          <cell r="V172"/>
-          <cell r="W172"/>
-          <cell r="X172"/>
-        </row>
-        <row r="173">
-          <cell r="D173"/>
-          <cell r="E173"/>
-          <cell r="F173"/>
-          <cell r="G173"/>
-          <cell r="H173"/>
-          <cell r="I173"/>
-          <cell r="J173"/>
-          <cell r="K173"/>
-          <cell r="L173"/>
-          <cell r="M173"/>
-          <cell r="N173"/>
-          <cell r="O173"/>
-          <cell r="P173"/>
-          <cell r="Q173"/>
-          <cell r="R173"/>
-          <cell r="S173"/>
-          <cell r="T173"/>
-          <cell r="U173"/>
-          <cell r="V173"/>
-          <cell r="W173"/>
-          <cell r="X173"/>
-        </row>
-        <row r="174">
-          <cell r="D174"/>
-          <cell r="E174"/>
-          <cell r="F174"/>
-          <cell r="G174"/>
-          <cell r="H174"/>
-          <cell r="I174"/>
-          <cell r="J174"/>
-          <cell r="K174"/>
-          <cell r="L174"/>
-          <cell r="M174"/>
-          <cell r="N174"/>
-          <cell r="O174"/>
-          <cell r="P174"/>
-          <cell r="Q174"/>
-          <cell r="R174"/>
-          <cell r="S174"/>
-          <cell r="T174"/>
-          <cell r="U174"/>
-          <cell r="V174"/>
-          <cell r="W174"/>
-          <cell r="X174"/>
-        </row>
-        <row r="175">
-          <cell r="D175"/>
-          <cell r="E175"/>
-          <cell r="F175"/>
-          <cell r="G175"/>
-          <cell r="H175"/>
-          <cell r="I175"/>
-          <cell r="J175"/>
-          <cell r="K175"/>
-          <cell r="L175"/>
-          <cell r="M175"/>
-          <cell r="N175"/>
-          <cell r="O175"/>
-          <cell r="P175"/>
-          <cell r="Q175"/>
-          <cell r="R175"/>
-          <cell r="S175"/>
-          <cell r="T175"/>
-          <cell r="U175"/>
-          <cell r="V175"/>
-          <cell r="W175"/>
-          <cell r="X175"/>
-        </row>
-        <row r="176">
-          <cell r="D176"/>
-          <cell r="E176"/>
-          <cell r="F176"/>
-          <cell r="G176"/>
-          <cell r="H176"/>
-          <cell r="I176"/>
-          <cell r="J176"/>
-          <cell r="K176"/>
-          <cell r="L176"/>
-          <cell r="M176"/>
-          <cell r="N176"/>
-          <cell r="O176"/>
-          <cell r="P176"/>
-          <cell r="Q176"/>
-          <cell r="R176"/>
-          <cell r="S176"/>
-          <cell r="T176"/>
-          <cell r="U176"/>
-          <cell r="V176"/>
-          <cell r="W176"/>
-          <cell r="X176"/>
-        </row>
-        <row r="177">
-          <cell r="D177"/>
-          <cell r="E177"/>
-          <cell r="F177"/>
-          <cell r="G177"/>
-          <cell r="H177"/>
-          <cell r="I177"/>
-          <cell r="J177"/>
-          <cell r="K177"/>
-          <cell r="L177"/>
-          <cell r="M177"/>
-          <cell r="N177"/>
-          <cell r="O177"/>
-          <cell r="P177"/>
-          <cell r="Q177"/>
-          <cell r="R177"/>
-          <cell r="S177"/>
-          <cell r="T177"/>
-          <cell r="U177"/>
-          <cell r="V177"/>
-          <cell r="W177"/>
-          <cell r="X177"/>
-        </row>
-        <row r="178">
-          <cell r="D178"/>
-          <cell r="E178"/>
-          <cell r="F178"/>
-          <cell r="G178"/>
-          <cell r="H178"/>
-          <cell r="I178"/>
-          <cell r="J178"/>
-          <cell r="K178"/>
-          <cell r="L178"/>
-          <cell r="M178"/>
-          <cell r="N178"/>
-          <cell r="O178"/>
-          <cell r="P178"/>
-          <cell r="Q178"/>
-          <cell r="R178"/>
-          <cell r="S178"/>
-          <cell r="T178"/>
-          <cell r="U178"/>
-          <cell r="V178"/>
-          <cell r="W178"/>
-          <cell r="X178"/>
-        </row>
-        <row r="179">
-          <cell r="D179"/>
-          <cell r="E179"/>
-          <cell r="F179"/>
-          <cell r="G179"/>
-          <cell r="H179"/>
-          <cell r="I179"/>
-          <cell r="J179"/>
-          <cell r="K179"/>
-          <cell r="L179"/>
-          <cell r="M179"/>
-          <cell r="N179"/>
-          <cell r="O179"/>
-          <cell r="P179"/>
-          <cell r="Q179"/>
-          <cell r="R179"/>
-          <cell r="S179"/>
-          <cell r="T179"/>
-          <cell r="U179"/>
-          <cell r="V179"/>
-          <cell r="W179"/>
-          <cell r="X179"/>
-        </row>
-        <row r="180">
-          <cell r="D180"/>
-          <cell r="E180"/>
-          <cell r="F180"/>
-          <cell r="G180"/>
-          <cell r="H180"/>
-          <cell r="I180"/>
-          <cell r="J180"/>
-          <cell r="K180"/>
-          <cell r="L180"/>
-          <cell r="M180"/>
-          <cell r="N180"/>
-          <cell r="O180"/>
-          <cell r="P180"/>
-          <cell r="Q180"/>
-          <cell r="R180"/>
-          <cell r="S180"/>
-          <cell r="T180"/>
-          <cell r="U180"/>
-          <cell r="V180"/>
-          <cell r="W180"/>
-          <cell r="X180"/>
-        </row>
-        <row r="181">
-          <cell r="D181"/>
-          <cell r="E181"/>
-          <cell r="F181"/>
-          <cell r="G181"/>
-          <cell r="H181"/>
-          <cell r="I181"/>
-          <cell r="J181"/>
-          <cell r="K181"/>
-          <cell r="L181"/>
-          <cell r="M181"/>
-          <cell r="N181"/>
-          <cell r="O181"/>
-          <cell r="P181"/>
-          <cell r="Q181"/>
-          <cell r="R181"/>
-          <cell r="S181"/>
-          <cell r="T181"/>
-          <cell r="U181"/>
-          <cell r="V181"/>
-          <cell r="W181"/>
-          <cell r="X181"/>
         </row>
       </sheetData>
     </sheetDataSet>
@@ -22408,7 +18636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2A118F-D7F3-5348-BECB-A41992F5CAD2}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -22418,10 +18646,10 @@
     <col min="5" max="5" width="6.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="10.83203125" style="1"/>
+    <col min="8" max="12" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>373</v>
       </c>
@@ -22453,13 +18681,16 @@
         <v>392</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>9</v>
       </c>
@@ -22498,15 +18729,16 @@
       <c r="J2" s="8" t="s">
         <v>443</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="5"/>
+      <c r="L2" s="9">
         <f>IF(J2="Yes",(H2*1500)/100,0)</f>
         <v>0</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -22532,7 +18764,7 @@
       </c>
       <c r="G3" s="7">
         <f>VLOOKUP(A3,[1]Games!$B$2:$K$398,9,FALSE)</f>
-        <v>0.44652162262184469</v>
+        <v>0.44652162262184492</v>
       </c>
       <c r="H3" s="7">
         <f>VLOOKUP(A3,[1]Games!$B$2:$K$398,7,FALSE)</f>
@@ -22545,12 +18777,13 @@
       <c r="J3" s="8" t="s">
         <v>443</v>
       </c>
-      <c r="K3" s="9">
-        <f t="shared" ref="K3" si="1">IF(J3="Yes",(H3*1500)/100,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K3" s="5"/>
+      <c r="L3" s="9">
+        <f t="shared" ref="L3" si="1">IF(J3="Yes",(H3*1500)/100,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -22568,11 +18801,11 @@
       </c>
       <c r="E4" s="5">
         <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,4,FALSE)</f>
-        <v>5.5829743724806304</v>
+        <v>5.257974372480632</v>
       </c>
       <c r="F4" s="5">
         <f>-VLOOKUP(A4,[2]Games!$A$2:$X$284,24,FALSE)</f>
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G4" s="7">
         <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,9,FALSE)</f>
@@ -22584,17 +18817,18 @@
       </c>
       <c r="I4" s="7">
         <f>VLOOKUP(A4,[1]Games!$B$2:$K$398,8,FALSE)/4</f>
-        <v>3.0921013343042949E-2</v>
+        <v>3.2949466586826175E-2</v>
       </c>
       <c r="J4" s="8" t="s">
         <v>443</v>
       </c>
-      <c r="K4" s="9">
-        <f t="shared" ref="K4:K9" si="3">IF(J4="Yes",(H4*1500)/100,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K4" s="5"/>
+      <c r="L4" s="9">
+        <f t="shared" ref="L4:L9" si="3">IF(J4="Yes",(H4*1500)/100,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -22633,12 +18867,13 @@
       <c r="J5" s="8" t="s">
         <v>443</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="5"/>
+      <c r="L5" s="9">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -22677,12 +18912,13 @@
       <c r="J6" s="8" t="s">
         <v>443</v>
       </c>
-      <c r="K6" s="9">
+      <c r="K6" s="5"/>
+      <c r="L6" s="9">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>14</v>
       </c>
@@ -22700,7 +18936,7 @@
       </c>
       <c r="E7" s="5">
         <f>VLOOKUP(A7,[1]Games!$B$2:$K$398,4,FALSE)</f>
-        <v>0.5490944982080217</v>
+        <v>0.54909449820802081</v>
       </c>
       <c r="F7" s="5">
         <f>-VLOOKUP(A7,[2]Games!$A$2:$X$284,24,FALSE)</f>
@@ -22708,7 +18944,7 @@
       </c>
       <c r="G7" s="7">
         <f>VLOOKUP(A7,[1]Games!$B$2:$K$398,9,FALSE)</f>
-        <v>0.28694196100801311</v>
+        <v>0.28694196100801289</v>
       </c>
       <c r="H7" s="7">
         <f>VLOOKUP(A7,[1]Games!$B$2:$K$398,7,FALSE)</f>
@@ -22721,12 +18957,13 @@
       <c r="J7" s="8" t="s">
         <v>443</v>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="5"/>
+      <c r="L7" s="9">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>15</v>
       </c>
@@ -22765,12 +19002,15 @@
       <c r="J8" s="8" t="s">
         <v>444</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="5">
+        <v>-111</v>
+      </c>
+      <c r="L8" s="9">
         <f t="shared" si="3"/>
         <v>0.7154130030427841</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -22809,12 +19049,13 @@
       <c r="J9" s="8" t="s">
         <v>443</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="5"/>
+      <c r="L9" s="9">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -22824,9 +19065,10 @@
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
       <c r="J10" s="8"/>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K10" s="5"/>
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
@@ -22836,9 +19078,10 @@
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="8"/>
-      <c r="K11" s="9"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K11" s="5"/>
+      <c r="L11" s="9"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -22848,9 +19091,10 @@
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
       <c r="J12" s="8"/>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K12" s="5"/>
+      <c r="L12" s="9"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
@@ -22860,9 +19104,10 @@
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
       <c r="J13" s="8"/>
-      <c r="K13" s="9"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K13" s="5"/>
+      <c r="L13" s="9"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -22872,9 +19117,10 @@
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
       <c r="J14" s="8"/>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K14" s="5"/>
+      <c r="L14" s="9"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
@@ -22884,9 +19130,10 @@
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
       <c r="J15" s="8"/>
-      <c r="K15" s="9"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K15" s="5"/>
+      <c r="L15" s="9"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
@@ -22896,9 +19143,10 @@
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
       <c r="J16" s="8"/>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K16" s="5"/>
+      <c r="L16" s="9"/>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
@@ -22908,9 +19156,10 @@
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
       <c r="J17" s="8"/>
-      <c r="K17" s="9"/>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K17" s="5"/>
+      <c r="L17" s="9"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
@@ -22920,9 +19169,10 @@
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
       <c r="J18" s="8"/>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K18" s="5"/>
+      <c r="L18" s="9"/>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -22932,9 +19182,10 @@
       <c r="H19" s="7"/>
       <c r="I19" s="7"/>
       <c r="J19" s="8"/>
-      <c r="K19" s="9"/>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K19" s="5"/>
+      <c r="L19" s="9"/>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
@@ -22944,9 +19195,10 @@
       <c r="H20" s="7"/>
       <c r="I20" s="7"/>
       <c r="J20" s="8"/>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K20" s="5"/>
+      <c r="L20" s="9"/>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -22956,9 +19208,10 @@
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
       <c r="J21" s="8"/>
-      <c r="K21" s="9"/>
-    </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K21" s="5"/>
+      <c r="L21" s="9"/>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
@@ -22968,9 +19221,10 @@
       <c r="H22" s="7"/>
       <c r="I22" s="7"/>
       <c r="J22" s="8"/>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K22" s="5"/>
+      <c r="L22" s="9"/>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
@@ -22980,9 +19234,10 @@
       <c r="H23" s="7"/>
       <c r="I23" s="7"/>
       <c r="J23" s="8"/>
-      <c r="K23" s="9"/>
-    </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K23" s="5"/>
+      <c r="L23" s="9"/>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
@@ -22992,9 +19247,10 @@
       <c r="H24" s="7"/>
       <c r="I24" s="7"/>
       <c r="J24" s="8"/>
-      <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K24" s="5"/>
+      <c r="L24" s="9"/>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
@@ -23004,9 +19260,10 @@
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
       <c r="J25" s="8"/>
-      <c r="K25" s="9"/>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K25" s="5"/>
+      <c r="L25" s="9"/>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
@@ -23016,9 +19273,10 @@
       <c r="H26" s="7"/>
       <c r="I26" s="7"/>
       <c r="J26" s="8"/>
-      <c r="K26" s="9"/>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K26" s="5"/>
+      <c r="L26" s="9"/>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -23028,9 +19286,10 @@
       <c r="H27" s="7"/>
       <c r="I27" s="7"/>
       <c r="J27" s="8"/>
-      <c r="K27" s="9"/>
-    </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K27" s="5"/>
+      <c r="L27" s="9"/>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
@@ -23040,9 +19299,10 @@
       <c r="H28" s="7"/>
       <c r="I28" s="7"/>
       <c r="J28" s="8"/>
-      <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K28" s="5"/>
+      <c r="L28" s="9"/>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -23052,9 +19312,10 @@
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
       <c r="J29" s="8"/>
-      <c r="K29" s="9"/>
-    </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K29" s="5"/>
+      <c r="L29" s="9"/>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
@@ -23064,9 +19325,10 @@
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="8"/>
-      <c r="K30" s="9"/>
-    </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K30" s="5"/>
+      <c r="L30" s="9"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
@@ -23076,9 +19338,10 @@
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="8"/>
-      <c r="K31" s="9"/>
-    </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K31" s="5"/>
+      <c r="L31" s="9"/>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
@@ -23088,9 +19351,10 @@
       <c r="H32" s="7"/>
       <c r="I32" s="7"/>
       <c r="J32" s="8"/>
-      <c r="K32" s="9"/>
-    </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K32" s="5"/>
+      <c r="L32" s="9"/>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
@@ -23100,9 +19364,10 @@
       <c r="H33" s="7"/>
       <c r="I33" s="7"/>
       <c r="J33" s="8"/>
-      <c r="K33" s="9"/>
-    </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K33" s="5"/>
+      <c r="L33" s="9"/>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
@@ -23112,9 +19377,10 @@
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="8"/>
-      <c r="K34" s="9"/>
-    </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K34" s="5"/>
+      <c r="L34" s="9"/>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
@@ -23124,9 +19390,10 @@
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="8"/>
-      <c r="K35" s="9"/>
-    </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K35" s="5"/>
+      <c r="L35" s="9"/>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
@@ -23136,9 +19403,10 @@
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="8"/>
-      <c r="K36" s="9"/>
-    </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="K36" s="5"/>
+      <c r="L36" s="9"/>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
@@ -23148,7 +19416,8 @@
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
       <c r="J37" s="8"/>
-      <c r="K37" s="9"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>